<commit_message>
Align task computation demand with reliability model
</commit_message>
<xml_diff>
--- a/data/task_parameters.xlsx
+++ b/data/task_parameters.xlsx
@@ -458,7 +458,7 @@
         <v>1.698676514770144</v>
       </c>
       <c r="C2" t="n">
-        <v>43.20759758426878</v>
+        <v>7</v>
       </c>
       <c r="D2" t="n">
         <v>0.99</v>
@@ -472,7 +472,7 @@
         <v>0.5576178793366848</v>
       </c>
       <c r="C3" t="n">
-        <v>43.38585708536767</v>
+        <v>23</v>
       </c>
       <c r="D3" t="n">
         <v>0.99</v>
@@ -486,7 +486,7 @@
         <v>1.124554743302174</v>
       </c>
       <c r="C4" t="n">
-        <v>27.45266138292878</v>
+        <v>7</v>
       </c>
       <c r="D4" t="n">
         <v>0.9999</v>
@@ -500,7 +500,7 @@
         <v>1.621772775239417</v>
       </c>
       <c r="C5" t="n">
-        <v>36.68641219189514</v>
+        <v>42</v>
       </c>
       <c r="D5" t="n">
         <v>0.9</v>
@@ -514,7 +514,7 @@
         <v>1.276891453942786</v>
       </c>
       <c r="C6" t="n">
-        <v>96.38144878048971</v>
+        <v>6</v>
       </c>
       <c r="D6" t="n">
         <v>0.999</v>
@@ -528,7 +528,7 @@
         <v>0.9167562239484524</v>
       </c>
       <c r="C7" t="n">
-        <v>55.13073435377007</v>
+        <v>43</v>
       </c>
       <c r="D7" t="n">
         <v>0.99</v>
@@ -542,7 +542,7 @@
         <v>1.125732881805666</v>
       </c>
       <c r="C8" t="n">
-        <v>75.08959796972462</v>
+        <v>31</v>
       </c>
       <c r="D8" t="n">
         <v>0.9</v>
@@ -556,7 +556,7 @@
         <v>0.8637911872546682</v>
       </c>
       <c r="C9" t="n">
-        <v>48.2333066780183</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
         <v>0.9999</v>
@@ -570,7 +570,7 @@
         <v>1.318929248634284</v>
       </c>
       <c r="C10" t="n">
-        <v>51.39147289948201</v>
+        <v>24</v>
       </c>
       <c r="D10" t="n">
         <v>0.9</v>
@@ -584,7 +584,7 @@
         <v>1.163224041631707</v>
       </c>
       <c r="C11" t="n">
-        <v>57.81777252679737</v>
+        <v>11</v>
       </c>
       <c r="D11" t="n">
         <v>0.999</v>
@@ -598,7 +598,7 @@
         <v>0.6171149990192427</v>
       </c>
       <c r="C12" t="n">
-        <v>60.20629815197702</v>
+        <v>40</v>
       </c>
       <c r="D12" t="n">
         <v>0.9999</v>
@@ -612,7 +612,7 @@
         <v>1.588839589559654</v>
       </c>
       <c r="C13" t="n">
-        <v>43.57610747977117</v>
+        <v>23</v>
       </c>
       <c r="D13" t="n">
         <v>0.999</v>
@@ -626,7 +626,7 @@
         <v>1.04376917576841</v>
       </c>
       <c r="C14" t="n">
-        <v>77.9882468342083</v>
+        <v>14</v>
       </c>
       <c r="D14" t="n">
         <v>0.999</v>
@@ -640,7 +640,7 @@
         <v>0.6063815335163489</v>
       </c>
       <c r="C15" t="n">
-        <v>24.09392907131769</v>
+        <v>16</v>
       </c>
       <c r="D15" t="n">
         <v>0.9</v>
@@ -654,7 +654,7 @@
         <v>0.5239759095260945</v>
       </c>
       <c r="C16" t="n">
-        <v>51.3555073720406</v>
+        <v>7</v>
       </c>
       <c r="D16" t="n">
         <v>0.999</v>
@@ -668,7 +668,7 @@
         <v>0.7325500786327677</v>
       </c>
       <c r="C17" t="n">
-        <v>53.78844418250332</v>
+        <v>7</v>
       </c>
       <c r="D17" t="n">
         <v>0.99</v>
@@ -682,7 +682,7 @@
         <v>1.500998025568986</v>
       </c>
       <c r="C18" t="n">
-        <v>49.05952338269637</v>
+        <v>14</v>
       </c>
       <c r="D18" t="n">
         <v>0.99</v>
@@ -696,7 +696,7 @@
         <v>1.865713256096655</v>
       </c>
       <c r="C19" t="n">
-        <v>21.31368435641481</v>
+        <v>37</v>
       </c>
       <c r="D19" t="n">
         <v>0.9</v>
@@ -710,7 +710,7 @@
         <v>1.617948301587924</v>
       </c>
       <c r="C20" t="n">
-        <v>56.52668008097017</v>
+        <v>45</v>
       </c>
       <c r="D20" t="n">
         <v>0.9</v>
@@ -724,7 +724,7 @@
         <v>1.091914683287179</v>
       </c>
       <c r="C21" t="n">
-        <v>44.30025813913874</v>
+        <v>19</v>
       </c>
       <c r="D21" t="n">
         <v>0.9999</v>
@@ -738,7 +738,7 @@
         <v>0.748173281639764</v>
       </c>
       <c r="C22" t="n">
-        <v>45.50457887351563</v>
+        <v>36</v>
       </c>
       <c r="D22" t="n">
         <v>0.9</v>
@@ -752,7 +752,7 @@
         <v>0.7023530680965311</v>
       </c>
       <c r="C23" t="n">
-        <v>55.02309588376541</v>
+        <v>44</v>
       </c>
       <c r="D23" t="n">
         <v>0.9</v>
@@ -766,7 +766,7 @@
         <v>1.28250873570704</v>
       </c>
       <c r="C24" t="n">
-        <v>52.18369220269612</v>
+        <v>10</v>
       </c>
       <c r="D24" t="n">
         <v>0.99</v>
@@ -780,7 +780,7 @@
         <v>0.5207435482617606</v>
       </c>
       <c r="C25" t="n">
-        <v>64.1433465628119</v>
+        <v>39</v>
       </c>
       <c r="D25" t="n">
         <v>0.9</v>
@@ -794,7 +794,7 @@
         <v>1.768814210603876</v>
       </c>
       <c r="C26" t="n">
-        <v>38.7105271323888</v>
+        <v>30</v>
       </c>
       <c r="D26" t="n">
         <v>0.9999</v>
@@ -808,7 +808,7 @@
         <v>1.933374127727371</v>
       </c>
       <c r="C27" t="n">
-        <v>47.15513362837858</v>
+        <v>17</v>
       </c>
       <c r="D27" t="n">
         <v>0.9999</v>
@@ -822,7 +822,7 @@
         <v>1.848292124784682</v>
       </c>
       <c r="C28" t="n">
-        <v>74.63638949869004</v>
+        <v>41</v>
       </c>
       <c r="D28" t="n">
         <v>0.99</v>
@@ -836,7 +836,7 @@
         <v>0.8606761119609709</v>
       </c>
       <c r="C29" t="n">
-        <v>26.42818394017014</v>
+        <v>20</v>
       </c>
       <c r="D29" t="n">
         <v>0.9</v>
@@ -850,7 +850,7 @@
         <v>1.435199088265653</v>
       </c>
       <c r="C30" t="n">
-        <v>37.81454435248695</v>
+        <v>34</v>
       </c>
       <c r="D30" t="n">
         <v>0.99</v>
@@ -864,7 +864,7 @@
         <v>1.200674143791567</v>
       </c>
       <c r="C31" t="n">
-        <v>11.55327504852977</v>
+        <v>32</v>
       </c>
       <c r="D31" t="n">
         <v>0.9999</v>
@@ -878,7 +878,7 @@
         <v>1.306239562439592</v>
       </c>
       <c r="C32" t="n">
-        <v>52.04782177376918</v>
+        <v>32</v>
       </c>
       <c r="D32" t="n">
         <v>0.999</v>
@@ -892,7 +892,7 @@
         <v>1.414121526506614</v>
       </c>
       <c r="C33" t="n">
-        <v>27.00002451712456</v>
+        <v>40</v>
       </c>
       <c r="D33" t="n">
         <v>0.999</v>
@@ -906,7 +906,7 @@
         <v>1.503259754869743</v>
       </c>
       <c r="C34" t="n">
-        <v>69.05176475181942</v>
+        <v>25</v>
       </c>
       <c r="D34" t="n">
         <v>0.99</v>
@@ -920,7 +920,7 @@
         <v>1.526822826982247</v>
       </c>
       <c r="C35" t="n">
-        <v>72.93728062802091</v>
+        <v>17</v>
       </c>
       <c r="D35" t="n">
         <v>0.9999</v>
@@ -934,7 +934,7 @@
         <v>0.5684495858010306</v>
       </c>
       <c r="C36" t="n">
-        <v>94.1892514143386</v>
+        <v>22</v>
       </c>
       <c r="D36" t="n">
         <v>0.99</v>
@@ -948,7 +948,7 @@
         <v>1.179773715471355</v>
       </c>
       <c r="C37" t="n">
-        <v>50.74555317850584</v>
+        <v>16</v>
       </c>
       <c r="D37" t="n">
         <v>0.99</v>
@@ -962,7 +962,7 @@
         <v>1.298240201487501</v>
       </c>
       <c r="C38" t="n">
-        <v>72.87509432348376</v>
+        <v>5</v>
       </c>
       <c r="D38" t="n">
         <v>0.999</v>
@@ -976,7 +976,7 @@
         <v>1.503696463389796</v>
       </c>
       <c r="C39" t="n">
-        <v>64.11347570332134</v>
+        <v>15</v>
       </c>
       <c r="D39" t="n">
         <v>0.99</v>
@@ -990,7 +990,7 @@
         <v>1.523658305587413</v>
       </c>
       <c r="C40" t="n">
-        <v>49.4848747688195</v>
+        <v>21</v>
       </c>
       <c r="D40" t="n">
         <v>0.9999</v>
@@ -1004,7 +1004,7 @@
         <v>1.223691777270608</v>
       </c>
       <c r="C41" t="n">
-        <v>40.61149836178698</v>
+        <v>44</v>
       </c>
       <c r="D41" t="n">
         <v>0.9</v>
@@ -1018,7 +1018,7 @@
         <v>1.034141742643207</v>
       </c>
       <c r="C42" t="n">
-        <v>55.49633659048928</v>
+        <v>6</v>
       </c>
       <c r="D42" t="n">
         <v>0.999</v>
@@ -1032,7 +1032,7 @@
         <v>0.8226734334855148</v>
       </c>
       <c r="C43" t="n">
-        <v>50.21304384090709</v>
+        <v>25</v>
       </c>
       <c r="D43" t="n">
         <v>0.99</v>
@@ -1046,7 +1046,7 @@
         <v>0.800146381586586</v>
       </c>
       <c r="C44" t="n">
-        <v>80.28697150155216</v>
+        <v>16</v>
       </c>
       <c r="D44" t="n">
         <v>0.99</v>
@@ -1060,7 +1060,7 @@
         <v>1.340370064244808</v>
       </c>
       <c r="C45" t="n">
-        <v>79.73797000587803</v>
+        <v>41</v>
       </c>
       <c r="D45" t="n">
         <v>0.99</v>
@@ -1074,7 +1074,7 @@
         <v>1.15931108163272</v>
       </c>
       <c r="C46" t="n">
-        <v>27.99943562898938</v>
+        <v>5</v>
       </c>
       <c r="D46" t="n">
         <v>0.9</v>
@@ -1088,7 +1088,7 @@
         <v>1.358026998454297</v>
       </c>
       <c r="C47" t="n">
-        <v>47.63495712009154</v>
+        <v>41</v>
       </c>
       <c r="D47" t="n">
         <v>0.9999</v>
@@ -1102,7 +1102,7 @@
         <v>0.7465153865434618</v>
       </c>
       <c r="C48" t="n">
-        <v>69.4777732317263</v>
+        <v>48</v>
       </c>
       <c r="D48" t="n">
         <v>0.9</v>
@@ -1116,7 +1116,7 @@
         <v>1.929676563507516</v>
       </c>
       <c r="C49" t="n">
-        <v>18.78144905959988</v>
+        <v>22</v>
       </c>
       <c r="D49" t="n">
         <v>0.999</v>
@@ -1130,7 +1130,7 @@
         <v>1.698174978067605</v>
       </c>
       <c r="C50" t="n">
-        <v>62.45478263683285</v>
+        <v>33</v>
       </c>
       <c r="D50" t="n">
         <v>0.9</v>
@@ -1144,7 +1144,7 @@
         <v>1.415739889683047</v>
       </c>
       <c r="C51" t="n">
-        <v>41.17089163372808</v>
+        <v>8</v>
       </c>
       <c r="D51" t="n">
         <v>0.999</v>
@@ -1158,7 +1158,7 @@
         <v>1.831453901303101</v>
       </c>
       <c r="C52" t="n">
-        <v>36.20911811232581</v>
+        <v>24</v>
       </c>
       <c r="D52" t="n">
         <v>0.999</v>
@@ -1172,7 +1172,7 @@
         <v>1.969558271783297</v>
       </c>
       <c r="C53" t="n">
-        <v>53.36755021048462</v>
+        <v>10</v>
       </c>
       <c r="D53" t="n">
         <v>0.99</v>
@@ -1186,7 +1186,7 @@
         <v>1.030740342586972</v>
       </c>
       <c r="C54" t="n">
-        <v>86.68081948680488</v>
+        <v>5</v>
       </c>
       <c r="D54" t="n">
         <v>0.9</v>
@@ -1200,7 +1200,7 @@
         <v>1.040929756161986</v>
       </c>
       <c r="C55" t="n">
-        <v>66.87614279594948</v>
+        <v>30</v>
       </c>
       <c r="D55" t="n">
         <v>0.999</v>
@@ -1214,7 +1214,7 @@
         <v>1.816948765493561</v>
       </c>
       <c r="C56" t="n">
-        <v>68.89653597946707</v>
+        <v>27</v>
       </c>
       <c r="D56" t="n">
         <v>0.99</v>
@@ -1228,7 +1228,7 @@
         <v>1.052073422806038</v>
       </c>
       <c r="C57" t="n">
-        <v>61.69922395929176</v>
+        <v>42</v>
       </c>
       <c r="D57" t="n">
         <v>0.99</v>
@@ -1242,7 +1242,7 @@
         <v>0.9040033107181582</v>
       </c>
       <c r="C58" t="n">
-        <v>54.15504567529959</v>
+        <v>15</v>
       </c>
       <c r="D58" t="n">
         <v>0.99</v>
@@ -1256,7 +1256,7 @@
         <v>0.9928927498253965</v>
       </c>
       <c r="C59" t="n">
-        <v>59.19308713179974</v>
+        <v>24</v>
       </c>
       <c r="D59" t="n">
         <v>0.99</v>
@@ -1270,7 +1270,7 @@
         <v>1.509078210389081</v>
       </c>
       <c r="C60" t="n">
-        <v>46.60421690982366</v>
+        <v>35</v>
       </c>
       <c r="D60" t="n">
         <v>0.9</v>
@@ -1284,7 +1284,7 @@
         <v>0.9862916350858244</v>
       </c>
       <c r="C61" t="n">
-        <v>57.55358370680607</v>
+        <v>23</v>
       </c>
       <c r="D61" t="n">
         <v>0.999</v>
@@ -1298,7 +1298,7 @@
         <v>1.141375014735014</v>
       </c>
       <c r="C62" t="n">
-        <v>52.07487047590578</v>
+        <v>45</v>
       </c>
       <c r="D62" t="n">
         <v>0.9999</v>
@@ -1312,7 +1312,7 @@
         <v>1.906647222467766</v>
       </c>
       <c r="C63" t="n">
-        <v>95.27992184950708</v>
+        <v>14</v>
       </c>
       <c r="D63" t="n">
         <v>0.999</v>
@@ -1326,7 +1326,7 @@
         <v>0.9521172516558767</v>
       </c>
       <c r="C64" t="n">
-        <v>69.17246069561165</v>
+        <v>11</v>
       </c>
       <c r="D64" t="n">
         <v>0.999</v>
@@ -1340,7 +1340,7 @@
         <v>0.8558423325051934</v>
       </c>
       <c r="C65" t="n">
-        <v>41.08058693360758</v>
+        <v>13</v>
       </c>
       <c r="D65" t="n">
         <v>0.99</v>
@@ -1354,7 +1354,7 @@
         <v>1.298123485843432</v>
       </c>
       <c r="C66" t="n">
-        <v>43.59202073570907</v>
+        <v>44</v>
       </c>
       <c r="D66" t="n">
         <v>0.99</v>
@@ -1368,7 +1368,7 @@
         <v>0.5713564090935292</v>
       </c>
       <c r="C67" t="n">
-        <v>44.53644711143514</v>
+        <v>9</v>
       </c>
       <c r="D67" t="n">
         <v>0.99</v>
@@ -1382,7 +1382,7 @@
         <v>1.972597559710513</v>
       </c>
       <c r="C68" t="n">
-        <v>51.41579418547523</v>
+        <v>26</v>
       </c>
       <c r="D68" t="n">
         <v>0.99</v>
@@ -1396,7 +1396,7 @@
         <v>1.430863916596355</v>
       </c>
       <c r="C69" t="n">
-        <v>34.08151122908987</v>
+        <v>18</v>
       </c>
       <c r="D69" t="n">
         <v>0.99</v>
@@ -1410,7 +1410,7 @@
         <v>1.146633986672343</v>
       </c>
       <c r="C70" t="n">
-        <v>54.65872410671282</v>
+        <v>15</v>
       </c>
       <c r="D70" t="n">
         <v>0.999</v>
@@ -1424,7 +1424,7 @@
         <v>1.816066291939203</v>
       </c>
       <c r="C71" t="n">
-        <v>66.48692590821491</v>
+        <v>26</v>
       </c>
       <c r="D71" t="n">
         <v>0.9999</v>
@@ -1438,7 +1438,7 @@
         <v>1.161652003910522</v>
       </c>
       <c r="C72" t="n">
-        <v>57.19324236092296</v>
+        <v>27</v>
       </c>
       <c r="D72" t="n">
         <v>0.9999</v>
@@ -1452,7 +1452,7 @@
         <v>0.5855852471050556</v>
       </c>
       <c r="C73" t="n">
-        <v>68.84173796027147</v>
+        <v>13</v>
       </c>
       <c r="D73" t="n">
         <v>0.999</v>
@@ -1466,7 +1466,7 @@
         <v>0.8087874084133323</v>
       </c>
       <c r="C74" t="n">
-        <v>54.13583146373279</v>
+        <v>20</v>
       </c>
       <c r="D74" t="n">
         <v>0.9999</v>
@@ -1480,7 +1480,7 @@
         <v>1.865168923911332</v>
       </c>
       <c r="C75" t="n">
-        <v>8.567289588645963</v>
+        <v>12</v>
       </c>
       <c r="D75" t="n">
         <v>0.9</v>
@@ -1494,7 +1494,7 @@
         <v>1.817678962718627</v>
       </c>
       <c r="C76" t="n">
-        <v>54.75334241138257</v>
+        <v>22</v>
       </c>
       <c r="D76" t="n">
         <v>0.999</v>
@@ -1508,7 +1508,7 @@
         <v>0.9642914675406724</v>
       </c>
       <c r="C77" t="n">
-        <v>52.81015271563107</v>
+        <v>15</v>
       </c>
       <c r="D77" t="n">
         <v>0.9999</v>
@@ -1522,7 +1522,7 @@
         <v>1.224190745013748</v>
       </c>
       <c r="C78" t="n">
-        <v>52.46396296696184</v>
+        <v>38</v>
       </c>
       <c r="D78" t="n">
         <v>0.9999</v>
@@ -1536,7 +1536,7 @@
         <v>1.132653855499087</v>
       </c>
       <c r="C79" t="n">
-        <v>58.79872928260366</v>
+        <v>11</v>
       </c>
       <c r="D79" t="n">
         <v>0.99</v>
@@ -1550,7 +1550,7 @@
         <v>1.441694714052209</v>
       </c>
       <c r="C80" t="n">
-        <v>18.72022139376082</v>
+        <v>50</v>
       </c>
       <c r="D80" t="n">
         <v>0.9</v>
@@ -1564,7 +1564,7 @@
         <v>0.888431824966925</v>
       </c>
       <c r="C81" t="n">
-        <v>43.90867391329789</v>
+        <v>20</v>
       </c>
       <c r="D81" t="n">
         <v>0.9999</v>
@@ -1578,7 +1578,7 @@
         <v>1.150241061134162</v>
       </c>
       <c r="C82" t="n">
-        <v>53.5985932196014</v>
+        <v>37</v>
       </c>
       <c r="D82" t="n">
         <v>0.99</v>
@@ -1592,7 +1592,7 @@
         <v>1.124274331781209</v>
       </c>
       <c r="C83" t="n">
-        <v>40.30209447778905</v>
+        <v>5</v>
       </c>
       <c r="D83" t="n">
         <v>0.99</v>
@@ -1606,7 +1606,7 @@
         <v>1.377181285809777</v>
       </c>
       <c r="C84" t="n">
-        <v>85.36821865802962</v>
+        <v>23</v>
       </c>
       <c r="D84" t="n">
         <v>0.999</v>
@@ -1620,7 +1620,7 @@
         <v>1.831081137486251</v>
       </c>
       <c r="C85" t="n">
-        <v>43.99412372367888</v>
+        <v>31</v>
       </c>
       <c r="D85" t="n">
         <v>0.9</v>
@@ -1634,7 +1634,7 @@
         <v>0.9514393938419983</v>
       </c>
       <c r="C86" t="n">
-        <v>40.39145421141154</v>
+        <v>35</v>
       </c>
       <c r="D86" t="n">
         <v>0.9999</v>
@@ -1648,7 +1648,7 @@
         <v>1.205959700518656</v>
       </c>
       <c r="C87" t="n">
-        <v>43.14945744753425</v>
+        <v>42</v>
       </c>
       <c r="D87" t="n">
         <v>0.999</v>
@@ -1662,7 +1662,7 @@
         <v>1.624691639598191</v>
       </c>
       <c r="C88" t="n">
-        <v>62.8857262773269</v>
+        <v>29</v>
       </c>
       <c r="D88" t="n">
         <v>0.9999</v>
@@ -1676,7 +1676,7 @@
         <v>1.325552594384797</v>
       </c>
       <c r="C89" t="n">
-        <v>60.93974912167573</v>
+        <v>6</v>
       </c>
       <c r="D89" t="n">
         <v>0.9999</v>
@@ -1690,7 +1690,7 @@
         <v>1.213340035311207</v>
       </c>
       <c r="C90" t="n">
-        <v>55.77546672427388</v>
+        <v>31</v>
       </c>
       <c r="D90" t="n">
         <v>0.9999</v>
@@ -1704,7 +1704,7 @@
         <v>1.534624620716951</v>
       </c>
       <c r="C91" t="n">
-        <v>68.77720052962201</v>
+        <v>16</v>
       </c>
       <c r="D91" t="n">
         <v>0.9</v>
@@ -1718,7 +1718,7 @@
         <v>1.997963898212609</v>
       </c>
       <c r="C92" t="n">
-        <v>51.18970735828495</v>
+        <v>13</v>
       </c>
       <c r="D92" t="n">
         <v>0.99</v>
@@ -1732,7 +1732,7 @@
         <v>1.566012214879641</v>
       </c>
       <c r="C93" t="n">
-        <v>69.84357131562507</v>
+        <v>29</v>
       </c>
       <c r="D93" t="n">
         <v>0.999</v>
@@ -1746,7 +1746,7 @@
         <v>1.903645965732959</v>
       </c>
       <c r="C94" t="n">
-        <v>48.4711112188855</v>
+        <v>42</v>
       </c>
       <c r="D94" t="n">
         <v>0.999</v>
@@ -1760,7 +1760,7 @@
         <v>1.245133191583559</v>
       </c>
       <c r="C95" t="n">
-        <v>38.38517172536942</v>
+        <v>49</v>
       </c>
       <c r="D95" t="n">
         <v>0.999</v>
@@ -1774,7 +1774,7 @@
         <v>1.017116826713074</v>
       </c>
       <c r="C96" t="n">
-        <v>98.94416185326097</v>
+        <v>46</v>
       </c>
       <c r="D96" t="n">
         <v>0.9999</v>
@@ -1788,7 +1788,7 @@
         <v>1.827822917119495</v>
       </c>
       <c r="C97" t="n">
-        <v>25.68209333658137</v>
+        <v>50</v>
       </c>
       <c r="D97" t="n">
         <v>0.9</v>
@@ -1802,7 +1802,7 @@
         <v>1.012730868611788</v>
       </c>
       <c r="C98" t="n">
-        <v>30.58917014906865</v>
+        <v>17</v>
       </c>
       <c r="D98" t="n">
         <v>0.999</v>
@@ -1816,7 +1816,7 @@
         <v>1.883181775512212</v>
       </c>
       <c r="C99" t="n">
-        <v>55.4789924474909</v>
+        <v>5</v>
       </c>
       <c r="D99" t="n">
         <v>0.9999</v>
@@ -1830,7 +1830,7 @@
         <v>1.418292648812512</v>
       </c>
       <c r="C100" t="n">
-        <v>25.94949736168169</v>
+        <v>49</v>
       </c>
       <c r="D100" t="n">
         <v>0.9</v>
@@ -1844,7 +1844,7 @@
         <v>0.9170233886763599</v>
       </c>
       <c r="C101" t="n">
-        <v>59.33338891114646</v>
+        <v>14</v>
       </c>
       <c r="D101" t="n">
         <v>0.9999</v>
@@ -1858,7 +1858,7 @@
         <v>0.9537779466483038</v>
       </c>
       <c r="C102" t="n">
-        <v>74.75354707657456</v>
+        <v>37</v>
       </c>
       <c r="D102" t="n">
         <v>0.9</v>
@@ -1872,7 +1872,7 @@
         <v>1.577314399725761</v>
       </c>
       <c r="C103" t="n">
-        <v>38.10131030109781</v>
+        <v>31</v>
       </c>
       <c r="D103" t="n">
         <v>0.9</v>
@@ -1886,7 +1886,7 @@
         <v>0.8845538199395837</v>
       </c>
       <c r="C104" t="n">
-        <v>59.09064323171441</v>
+        <v>49</v>
       </c>
       <c r="D104" t="n">
         <v>0.99</v>
@@ -1900,7 +1900,7 @@
         <v>1.986382241334534</v>
       </c>
       <c r="C105" t="n">
-        <v>45.76409327869553</v>
+        <v>37</v>
       </c>
       <c r="D105" t="n">
         <v>0.9999</v>
@@ -1914,7 +1914,7 @@
         <v>1.917266514357731</v>
       </c>
       <c r="C106" t="n">
-        <v>47.79058529410705</v>
+        <v>27</v>
       </c>
       <c r="D106" t="n">
         <v>0.9999</v>
@@ -1928,7 +1928,7 @@
         <v>0.9772057199456969</v>
       </c>
       <c r="C107" t="n">
-        <v>54.99188807458597</v>
+        <v>20</v>
       </c>
       <c r="D107" t="n">
         <v>0.9</v>
@@ -1942,7 +1942,7 @@
         <v>0.8832316178677049</v>
       </c>
       <c r="C108" t="n">
-        <v>55.97322148583545</v>
+        <v>48</v>
       </c>
       <c r="D108" t="n">
         <v>0.9</v>
@@ -1956,7 +1956,7 @@
         <v>1.475667183557569</v>
       </c>
       <c r="C109" t="n">
-        <v>54.07640908246629</v>
+        <v>35</v>
       </c>
       <c r="D109" t="n">
         <v>0.9999</v>
@@ -1970,7 +1970,7 @@
         <v>1.193530399564723</v>
       </c>
       <c r="C110" t="n">
-        <v>77.2673948909937</v>
+        <v>20</v>
       </c>
       <c r="D110" t="n">
         <v>0.9</v>
@@ -1984,7 +1984,7 @@
         <v>1.526682248403668</v>
       </c>
       <c r="C111" t="n">
-        <v>12.33299322717335</v>
+        <v>22</v>
       </c>
       <c r="D111" t="n">
         <v>0.9999</v>
@@ -1998,7 +1998,7 @@
         <v>1.99592970650501</v>
       </c>
       <c r="C112" t="n">
-        <v>32.10974931541395</v>
+        <v>50</v>
       </c>
       <c r="D112" t="n">
         <v>0.999</v>
@@ -2012,7 +2012,7 @@
         <v>0.5265638021424695</v>
       </c>
       <c r="C113" t="n">
-        <v>67.73622975761094</v>
+        <v>29</v>
       </c>
       <c r="D113" t="n">
         <v>0.9999</v>
@@ -2026,7 +2026,7 @@
         <v>0.5161931264924058</v>
       </c>
       <c r="C114" t="n">
-        <v>66.40356718027326</v>
+        <v>50</v>
       </c>
       <c r="D114" t="n">
         <v>0.99</v>
@@ -2040,7 +2040,7 @@
         <v>1.967253588335947</v>
       </c>
       <c r="C115" t="n">
-        <v>31.78790631655901</v>
+        <v>22</v>
       </c>
       <c r="D115" t="n">
         <v>0.9999</v>
@@ -2054,7 +2054,7 @@
         <v>1.89615348425003</v>
       </c>
       <c r="C116" t="n">
-        <v>64.37726779703684</v>
+        <v>39</v>
       </c>
       <c r="D116" t="n">
         <v>0.9999</v>
@@ -2068,7 +2068,7 @@
         <v>0.6965759756239653</v>
       </c>
       <c r="C117" t="n">
-        <v>53.40776155781828</v>
+        <v>38</v>
       </c>
       <c r="D117" t="n">
         <v>0.9</v>
@@ -2082,7 +2082,7 @@
         <v>1.941117476679422</v>
       </c>
       <c r="C118" t="n">
-        <v>76.25004893712321</v>
+        <v>39</v>
       </c>
       <c r="D118" t="n">
         <v>0.99</v>
@@ -2096,7 +2096,7 @@
         <v>0.9390548602461679</v>
       </c>
       <c r="C119" t="n">
-        <v>72.66476000723722</v>
+        <v>16</v>
       </c>
       <c r="D119" t="n">
         <v>0.999</v>
@@ -2110,7 +2110,7 @@
         <v>1.005056755933833</v>
       </c>
       <c r="C120" t="n">
-        <v>55.47989910062199</v>
+        <v>50</v>
       </c>
       <c r="D120" t="n">
         <v>0.9999</v>
@@ -2124,7 +2124,7 @@
         <v>1.57653010894631</v>
       </c>
       <c r="C121" t="n">
-        <v>61.25705195827475</v>
+        <v>36</v>
       </c>
       <c r="D121" t="n">
         <v>0.9999</v>
@@ -2138,7 +2138,7 @@
         <v>1.138993162495187</v>
       </c>
       <c r="C122" t="n">
-        <v>33.63993991992791</v>
+        <v>31</v>
       </c>
       <c r="D122" t="n">
         <v>0.99</v>
@@ -2152,7 +2152,7 @@
         <v>1.210173278683276</v>
       </c>
       <c r="C123" t="n">
-        <v>37.77805304550698</v>
+        <v>23</v>
       </c>
       <c r="D123" t="n">
         <v>0.99</v>
@@ -2166,7 +2166,7 @@
         <v>1.590989166316217</v>
       </c>
       <c r="C124" t="n">
-        <v>61.57428809194288</v>
+        <v>29</v>
       </c>
       <c r="D124" t="n">
         <v>0.9</v>
@@ -2180,7 +2180,7 @@
         <v>0.6343737052454252</v>
       </c>
       <c r="C125" t="n">
-        <v>59.34728818910371</v>
+        <v>24</v>
       </c>
       <c r="D125" t="n">
         <v>0.9</v>
@@ -2194,7 +2194,7 @@
         <v>1.768735631079944</v>
       </c>
       <c r="C126" t="n">
-        <v>59.3527919898704</v>
+        <v>32</v>
       </c>
       <c r="D126" t="n">
         <v>0.999</v>
@@ -2208,7 +2208,7 @@
         <v>0.8723914376346985</v>
       </c>
       <c r="C127" t="n">
-        <v>47.89550907575663</v>
+        <v>40</v>
       </c>
       <c r="D127" t="n">
         <v>0.9999</v>
@@ -2222,7 +2222,7 @@
         <v>0.68677596232893</v>
       </c>
       <c r="C128" t="n">
-        <v>87.62819238440366</v>
+        <v>6</v>
       </c>
       <c r="D128" t="n">
         <v>0.999</v>
@@ -2236,7 +2236,7 @@
         <v>1.920396836566512</v>
       </c>
       <c r="C129" t="n">
-        <v>60.22400849114594</v>
+        <v>38</v>
       </c>
       <c r="D129" t="n">
         <v>0.999</v>
@@ -2250,7 +2250,7 @@
         <v>1.909367759380076</v>
       </c>
       <c r="C130" t="n">
-        <v>55.5412462608636</v>
+        <v>40</v>
       </c>
       <c r="D130" t="n">
         <v>0.9999</v>
@@ -2264,7 +2264,7 @@
         <v>1.393498512084533</v>
       </c>
       <c r="C131" t="n">
-        <v>58.402427945288</v>
+        <v>5</v>
       </c>
       <c r="D131" t="n">
         <v>0.9</v>
@@ -2278,7 +2278,7 @@
         <v>1.187596167398222</v>
       </c>
       <c r="C132" t="n">
-        <v>35.57338683031903</v>
+        <v>23</v>
       </c>
       <c r="D132" t="n">
         <v>0.999</v>
@@ -2292,7 +2292,7 @@
         <v>1.272934462939539</v>
       </c>
       <c r="C133" t="n">
-        <v>35.6998408361998</v>
+        <v>48</v>
       </c>
       <c r="D133" t="n">
         <v>0.99</v>
@@ -2306,7 +2306,7 @@
         <v>1.153128796728891</v>
       </c>
       <c r="C134" t="n">
-        <v>28.28236827025106</v>
+        <v>15</v>
       </c>
       <c r="D134" t="n">
         <v>0.99</v>
@@ -2320,7 +2320,7 @@
         <v>1.16045611412061</v>
       </c>
       <c r="C135" t="n">
-        <v>43.97417121229151</v>
+        <v>33</v>
       </c>
       <c r="D135" t="n">
         <v>0.9</v>
@@ -2334,7 +2334,7 @@
         <v>1.014730722566602</v>
       </c>
       <c r="C136" t="n">
-        <v>32.6642947372342</v>
+        <v>34</v>
       </c>
       <c r="D136" t="n">
         <v>0.999</v>
@@ -2348,7 +2348,7 @@
         <v>1.376458654732497</v>
       </c>
       <c r="C137" t="n">
-        <v>59.32849460019946</v>
+        <v>8</v>
       </c>
       <c r="D137" t="n">
         <v>0.999</v>
@@ -2362,7 +2362,7 @@
         <v>0.9158407099198769</v>
       </c>
       <c r="C138" t="n">
-        <v>53.79870291338703</v>
+        <v>37</v>
       </c>
       <c r="D138" t="n">
         <v>0.999</v>
@@ -2376,7 +2376,7 @@
         <v>1.161024498520936</v>
       </c>
       <c r="C139" t="n">
-        <v>51.07101703821254</v>
+        <v>26</v>
       </c>
       <c r="D139" t="n">
         <v>0.9</v>
@@ -2390,7 +2390,7 @@
         <v>0.5691682785320457</v>
       </c>
       <c r="C140" t="n">
-        <v>59.44097895331267</v>
+        <v>29</v>
       </c>
       <c r="D140" t="n">
         <v>0.999</v>
@@ -2404,7 +2404,7 @@
         <v>0.558185544582529</v>
       </c>
       <c r="C141" t="n">
-        <v>45.6646095015544</v>
+        <v>28</v>
       </c>
       <c r="D141" t="n">
         <v>0.9999</v>
@@ -2418,7 +2418,7 @@
         <v>1.067330561012164</v>
       </c>
       <c r="C142" t="n">
-        <v>47.02182939587593</v>
+        <v>35</v>
       </c>
       <c r="D142" t="n">
         <v>0.99</v>
@@ -2432,7 +2432,7 @@
         <v>1.879025263275386</v>
       </c>
       <c r="C143" t="n">
-        <v>56.52014523281619</v>
+        <v>5</v>
       </c>
       <c r="D143" t="n">
         <v>0.99</v>
@@ -2446,7 +2446,7 @@
         <v>1.425020254339325</v>
       </c>
       <c r="C144" t="n">
-        <v>18.64237593166486</v>
+        <v>21</v>
       </c>
       <c r="D144" t="n">
         <v>0.999</v>
@@ -2460,7 +2460,7 @@
         <v>1.372806673584253</v>
       </c>
       <c r="C145" t="n">
-        <v>41.60180208730131</v>
+        <v>38</v>
       </c>
       <c r="D145" t="n">
         <v>0.99</v>
@@ -2474,7 +2474,7 @@
         <v>0.8007931175918177</v>
       </c>
       <c r="C146" t="n">
-        <v>82.7650811433617</v>
+        <v>36</v>
       </c>
       <c r="D146" t="n">
         <v>0.9</v>
@@ -2488,7 +2488,7 @@
         <v>1.440880270175235</v>
       </c>
       <c r="C147" t="n">
-        <v>42.37732900086705</v>
+        <v>34</v>
       </c>
       <c r="D147" t="n">
         <v>0.999</v>
@@ -2502,7 +2502,7 @@
         <v>0.715362962414009</v>
       </c>
       <c r="C148" t="n">
-        <v>49.95398679298959</v>
+        <v>6</v>
       </c>
       <c r="D148" t="n">
         <v>0.9</v>
@@ -2516,7 +2516,7 @@
         <v>1.560571204256596</v>
       </c>
       <c r="C149" t="n">
-        <v>38.18412672813696</v>
+        <v>36</v>
       </c>
       <c r="D149" t="n">
         <v>0.999</v>
@@ -2530,7 +2530,7 @@
         <v>1.846820848597533</v>
       </c>
       <c r="C150" t="n">
-        <v>51.8560884160152</v>
+        <v>34</v>
       </c>
       <c r="D150" t="n">
         <v>0.999</v>
@@ -2544,7 +2544,7 @@
         <v>0.8290130927646091</v>
       </c>
       <c r="C151" t="n">
-        <v>29.7875634683097</v>
+        <v>17</v>
       </c>
       <c r="D151" t="n">
         <v>0.9</v>
@@ -2558,7 +2558,7 @@
         <v>1.621975929178317</v>
       </c>
       <c r="C152" t="n">
-        <v>54.10473410883696</v>
+        <v>7</v>
       </c>
       <c r="D152" t="n">
         <v>0.99</v>
@@ -2572,7 +2572,7 @@
         <v>1.826859764671628</v>
       </c>
       <c r="C153" t="n">
-        <v>29.66099402171883</v>
+        <v>38</v>
       </c>
       <c r="D153" t="n">
         <v>0.99</v>
@@ -2586,7 +2586,7 @@
         <v>1.020755919076118</v>
       </c>
       <c r="C154" t="n">
-        <v>57.0871940191464</v>
+        <v>35</v>
       </c>
       <c r="D154" t="n">
         <v>0.999</v>
@@ -2600,7 +2600,7 @@
         <v>1.462888622687835</v>
       </c>
       <c r="C155" t="n">
-        <v>23.81428370738922</v>
+        <v>27</v>
       </c>
       <c r="D155" t="n">
         <v>0.9999</v>
@@ -2614,7 +2614,7 @@
         <v>0.7011151675491456</v>
       </c>
       <c r="C156" t="n">
-        <v>48.11775373375345</v>
+        <v>26</v>
       </c>
       <c r="D156" t="n">
         <v>0.999</v>
@@ -2628,7 +2628,7 @@
         <v>1.21156168911754</v>
       </c>
       <c r="C157" t="n">
-        <v>46.36413000420836</v>
+        <v>41</v>
       </c>
       <c r="D157" t="n">
         <v>0.99</v>
@@ -2642,7 +2642,7 @@
         <v>1.959051147849327</v>
       </c>
       <c r="C158" t="n">
-        <v>32.01678878891607</v>
+        <v>17</v>
       </c>
       <c r="D158" t="n">
         <v>0.999</v>
@@ -2656,7 +2656,7 @@
         <v>1.59819000355857</v>
       </c>
       <c r="C159" t="n">
-        <v>66.33555871283548</v>
+        <v>12</v>
       </c>
       <c r="D159" t="n">
         <v>0.9999</v>
@@ -2670,7 +2670,7 @@
         <v>1.029338817444233</v>
       </c>
       <c r="C160" t="n">
-        <v>40.86823229046978</v>
+        <v>15</v>
       </c>
       <c r="D160" t="n">
         <v>0.9999</v>
@@ -2684,7 +2684,7 @@
         <v>1.110467212912065</v>
       </c>
       <c r="C161" t="n">
-        <v>63.04176689852675</v>
+        <v>32</v>
       </c>
       <c r="D161" t="n">
         <v>0.9</v>
@@ -2698,7 +2698,7 @@
         <v>1.518168198151698</v>
       </c>
       <c r="C162" t="n">
-        <v>45.01544938245973</v>
+        <v>5</v>
       </c>
       <c r="D162" t="n">
         <v>0.9999</v>
@@ -2712,7 +2712,7 @@
         <v>0.6461838780613436</v>
       </c>
       <c r="C163" t="n">
-        <v>46.94076825568083</v>
+        <v>12</v>
       </c>
       <c r="D163" t="n">
         <v>0.99</v>
@@ -2726,7 +2726,7 @@
         <v>1.478815136842968</v>
       </c>
       <c r="C164" t="n">
-        <v>80.96459994383044</v>
+        <v>22</v>
       </c>
       <c r="D164" t="n">
         <v>0.9</v>
@@ -2740,7 +2740,7 @@
         <v>1.43791051418215</v>
       </c>
       <c r="C165" t="n">
-        <v>55.70445243448228</v>
+        <v>46</v>
       </c>
       <c r="D165" t="n">
         <v>0.999</v>
@@ -2754,7 +2754,7 @@
         <v>1.970451205844075</v>
       </c>
       <c r="C166" t="n">
-        <v>60.22060361378609</v>
+        <v>44</v>
       </c>
       <c r="D166" t="n">
         <v>0.99</v>
@@ -2768,7 +2768,7 @@
         <v>0.6165587144900581</v>
       </c>
       <c r="C167" t="n">
-        <v>35.52447847044257</v>
+        <v>50</v>
       </c>
       <c r="D167" t="n">
         <v>0.999</v>
@@ -2782,7 +2782,7 @@
         <v>1.777549109504937</v>
       </c>
       <c r="C168" t="n">
-        <v>74.83796044440696</v>
+        <v>43</v>
       </c>
       <c r="D168" t="n">
         <v>0.9999</v>
@@ -2796,7 +2796,7 @@
         <v>1.923435722078754</v>
       </c>
       <c r="C169" t="n">
-        <v>35.91062707574415</v>
+        <v>12</v>
       </c>
       <c r="D169" t="n">
         <v>0.999</v>
@@ -2810,7 +2810,7 @@
         <v>0.50410556434063</v>
       </c>
       <c r="C170" t="n">
-        <v>41.07876824153396</v>
+        <v>28</v>
       </c>
       <c r="D170" t="n">
         <v>0.9999</v>
@@ -2824,7 +2824,7 @@
         <v>0.682665623139759</v>
       </c>
       <c r="C171" t="n">
-        <v>27.83349922363659</v>
+        <v>20</v>
       </c>
       <c r="D171" t="n">
         <v>0.999</v>
@@ -2838,7 +2838,7 @@
         <v>1.013140134936704</v>
       </c>
       <c r="C172" t="n">
-        <v>10.60510472593611</v>
+        <v>14</v>
       </c>
       <c r="D172" t="n">
         <v>0.999</v>
@@ -2852,7 +2852,7 @@
         <v>1.827315687959412</v>
       </c>
       <c r="C173" t="n">
-        <v>56.57070459279413</v>
+        <v>43</v>
       </c>
       <c r="D173" t="n">
         <v>0.9999</v>
@@ -2866,7 +2866,7 @@
         <v>1.713205254747983</v>
       </c>
       <c r="C174" t="n">
-        <v>36.25296257009146</v>
+        <v>12</v>
       </c>
       <c r="D174" t="n">
         <v>0.9</v>
@@ -2880,7 +2880,7 @@
         <v>1.45624265265026</v>
       </c>
       <c r="C175" t="n">
-        <v>46.00948760840934</v>
+        <v>37</v>
       </c>
       <c r="D175" t="n">
         <v>0.9999</v>
@@ -2894,7 +2894,7 @@
         <v>0.5195565980853729</v>
       </c>
       <c r="C176" t="n">
-        <v>64.98581463610341</v>
+        <v>38</v>
       </c>
       <c r="D176" t="n">
         <v>0.9</v>
@@ -2908,7 +2908,7 @@
         <v>1.412912890468327</v>
       </c>
       <c r="C177" t="n">
-        <v>39.57041138402937</v>
+        <v>29</v>
       </c>
       <c r="D177" t="n">
         <v>0.99</v>
@@ -2922,7 +2922,7 @@
         <v>1.943389560641203</v>
       </c>
       <c r="C178" t="n">
-        <v>38.26119121400266</v>
+        <v>5</v>
       </c>
       <c r="D178" t="n">
         <v>0.9</v>
@@ -2936,7 +2936,7 @@
         <v>1.566008595031556</v>
       </c>
       <c r="C179" t="n">
-        <v>39.40324060927303</v>
+        <v>22</v>
       </c>
       <c r="D179" t="n">
         <v>0.9</v>
@@ -2950,7 +2950,7 @@
         <v>1.421481188363827</v>
       </c>
       <c r="C180" t="n">
-        <v>48.43212035316666</v>
+        <v>40</v>
       </c>
       <c r="D180" t="n">
         <v>0.99</v>
@@ -2964,7 +2964,7 @@
         <v>0.9661528785946254</v>
       </c>
       <c r="C181" t="n">
-        <v>96.49696595745532</v>
+        <v>32</v>
       </c>
       <c r="D181" t="n">
         <v>0.99</v>
@@ -2978,7 +2978,7 @@
         <v>1.016994233974312</v>
       </c>
       <c r="C182" t="n">
-        <v>41.70215136698815</v>
+        <v>33</v>
       </c>
       <c r="D182" t="n">
         <v>0.9</v>
@@ -2992,7 +2992,7 @@
         <v>1.289320399650121</v>
       </c>
       <c r="C183" t="n">
-        <v>68.45673375956804</v>
+        <v>21</v>
       </c>
       <c r="D183" t="n">
         <v>0.9</v>
@@ -3006,7 +3006,7 @@
         <v>0.8684840279545238</v>
       </c>
       <c r="C184" t="n">
-        <v>51.49323544861909</v>
+        <v>21</v>
       </c>
       <c r="D184" t="n">
         <v>0.999</v>
@@ -3020,7 +3020,7 @@
         <v>0.5233041138229977</v>
       </c>
       <c r="C185" t="n">
-        <v>59.34093572922665</v>
+        <v>18</v>
       </c>
       <c r="D185" t="n">
         <v>0.9999</v>
@@ -3034,7 +3034,7 @@
         <v>1.080886887873118</v>
       </c>
       <c r="C186" t="n">
-        <v>67.83919761244347</v>
+        <v>21</v>
       </c>
       <c r="D186" t="n">
         <v>0.9</v>
@@ -3048,7 +3048,7 @@
         <v>1.936002494005718</v>
       </c>
       <c r="C187" t="n">
-        <v>30.02472658904182</v>
+        <v>35</v>
       </c>
       <c r="D187" t="n">
         <v>0.9</v>
@@ -3062,7 +3062,7 @@
         <v>0.8823253989818636</v>
       </c>
       <c r="C188" t="n">
-        <v>50.53243129360188</v>
+        <v>10</v>
       </c>
       <c r="D188" t="n">
         <v>0.9999</v>
@@ -3076,7 +3076,7 @@
         <v>0.5888615131268994</v>
       </c>
       <c r="C189" t="n">
-        <v>37.10279117957653</v>
+        <v>13</v>
       </c>
       <c r="D189" t="n">
         <v>0.99</v>
@@ -3090,7 +3090,7 @@
         <v>1.493961165977075</v>
       </c>
       <c r="C190" t="n">
-        <v>84.60916806538907</v>
+        <v>23</v>
       </c>
       <c r="D190" t="n">
         <v>0.9</v>
@@ -3104,7 +3104,7 @@
         <v>1.846857262790149</v>
       </c>
       <c r="C191" t="n">
-        <v>51.33048636029659</v>
+        <v>19</v>
       </c>
       <c r="D191" t="n">
         <v>0.9999</v>
@@ -3118,7 +3118,7 @@
         <v>0.80785866874114</v>
       </c>
       <c r="C192" t="n">
-        <v>30.99292366373328</v>
+        <v>25</v>
       </c>
       <c r="D192" t="n">
         <v>0.9999</v>
@@ -3132,7 +3132,7 @@
         <v>1.550979765374794</v>
       </c>
       <c r="C193" t="n">
-        <v>30.96494662908491</v>
+        <v>13</v>
       </c>
       <c r="D193" t="n">
         <v>0.99</v>
@@ -3146,7 +3146,7 @@
         <v>1.038987919243236</v>
       </c>
       <c r="C194" t="n">
-        <v>58.23712976094647</v>
+        <v>9</v>
       </c>
       <c r="D194" t="n">
         <v>0.9</v>
@@ -3160,7 +3160,7 @@
         <v>1.264389791626048</v>
       </c>
       <c r="C195" t="n">
-        <v>30.91992531690555</v>
+        <v>46</v>
       </c>
       <c r="D195" t="n">
         <v>0.9</v>
@@ -3174,7 +3174,7 @@
         <v>0.7213409319196464</v>
       </c>
       <c r="C196" t="n">
-        <v>38.28294551366284</v>
+        <v>27</v>
       </c>
       <c r="D196" t="n">
         <v>0.99</v>
@@ -3188,7 +3188,7 @@
         <v>1.784902233608911</v>
       </c>
       <c r="C197" t="n">
-        <v>69.01566878980147</v>
+        <v>44</v>
       </c>
       <c r="D197" t="n">
         <v>0.999</v>
@@ -3202,7 +3202,7 @@
         <v>1.44872661437035</v>
       </c>
       <c r="C198" t="n">
-        <v>60.56783139759938</v>
+        <v>27</v>
       </c>
       <c r="D198" t="n">
         <v>0.999</v>
@@ -3216,7 +3216,7 @@
         <v>1.464910533836621</v>
       </c>
       <c r="C199" t="n">
-        <v>43.66447095291823</v>
+        <v>45</v>
       </c>
       <c r="D199" t="n">
         <v>0.9999</v>
@@ -3230,7 +3230,7 @@
         <v>1.879986701906027</v>
       </c>
       <c r="C200" t="n">
-        <v>85.42407309850805</v>
+        <v>22</v>
       </c>
       <c r="D200" t="n">
         <v>0.9</v>
@@ -3244,7 +3244,7 @@
         <v>1.258948347352817</v>
       </c>
       <c r="C201" t="n">
-        <v>40.37192940527918</v>
+        <v>40</v>
       </c>
       <c r="D201" t="n">
         <v>0.9999</v>

</xml_diff>

<commit_message>
Generate task reliability requirement profiles
</commit_message>
<xml_diff>
--- a/data/task_parameters.xlsx
+++ b/data/task_parameters.xlsx
@@ -460,7 +460,9 @@
       <c r="C2" t="n">
         <v>53.67919023703534</v>
       </c>
-      <c r="D2" t="inlineStr"/>
+      <c r="D2" t="n">
+        <v>0.9916104133230789</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -472,7 +474,9 @@
       <c r="C3" t="n">
         <v>34.75107857408746</v>
       </c>
-      <c r="D3" t="inlineStr"/>
+      <c r="D3" t="n">
+        <v>0.9957592184914363</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -484,7 +488,9 @@
       <c r="C4" t="n">
         <v>42.60628635542257</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>0.9942054156102914</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -496,7 +502,9 @@
       <c r="C5" t="n">
         <v>33.48190127293107</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="D5" t="n">
+        <v>0.9933345047439724</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -508,7 +516,9 @@
       <c r="C6" t="n">
         <v>45.23196171646185</v>
       </c>
-      <c r="D6" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>0.9931942560087869</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -520,7 +530,9 @@
       <c r="C7" t="n">
         <v>42.32918817317876</v>
       </c>
-      <c r="D7" t="inlineStr"/>
+      <c r="D7" t="n">
+        <v>0.9971146642126794</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -532,7 +544,9 @@
       <c r="C8" t="n">
         <v>44.44014536248625</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>0.9981462945300945</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -544,7 +558,9 @@
       <c r="C9" t="n">
         <v>47.94897151388241</v>
       </c>
-      <c r="D9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>0.9915961787264075</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -556,7 +572,9 @@
       <c r="C10" t="n">
         <v>44.64165636479374</v>
       </c>
-      <c r="D10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>0.9958750632241662</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -568,7 +586,9 @@
       <c r="C11" t="n">
         <v>28.02194103187311</v>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>0.9926847249062001</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -580,7 +600,9 @@
       <c r="C12" t="n">
         <v>50.49475649543508</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>0.9987026598014616</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -592,7 +614,9 @@
       <c r="C13" t="n">
         <v>40.71306000432234</v>
       </c>
-      <c r="D13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>0.9982786514448355</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -604,7 +628,9 @@
       <c r="C14" t="n">
         <v>47.09592044693731</v>
       </c>
-      <c r="D14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>0.9957228372373018</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -616,7 +642,9 @@
       <c r="C15" t="n">
         <v>62.52548385599771</v>
       </c>
-      <c r="D15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>0.9967745888737117</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -628,7 +656,9 @@
       <c r="C16" t="n">
         <v>54.260886173613</v>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>0.9946363832669012</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -640,7 +670,9 @@
       <c r="C17" t="n">
         <v>60.50559856437604</v>
       </c>
-      <c r="D17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>0.9974330573253801</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -652,7 +684,9 @@
       <c r="C18" t="n">
         <v>71.04614060419865</v>
       </c>
-      <c r="D18" t="inlineStr"/>
+      <c r="D18" t="n">
+        <v>0.994035424908601</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -664,7 +698,9 @@
       <c r="C19" t="n">
         <v>58.55154095134137</v>
       </c>
-      <c r="D19" t="inlineStr"/>
+      <c r="D19" t="n">
+        <v>0.9930493120798238</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -676,7 +712,9 @@
       <c r="C20" t="n">
         <v>51.66508863793452</v>
       </c>
-      <c r="D20" t="inlineStr"/>
+      <c r="D20" t="n">
+        <v>0.9925010929395014</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -688,7 +726,9 @@
       <c r="C21" t="n">
         <v>78.40138622491851</v>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="D21" t="n">
+        <v>0.9920369975115906</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -700,7 +740,9 @@
       <c r="C22" t="n">
         <v>48.7360258336366</v>
       </c>
-      <c r="D22" t="inlineStr"/>
+      <c r="D22" t="n">
+        <v>0.9947323515901072</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -712,7 +754,9 @@
       <c r="C23" t="n">
         <v>49.85244703050946</v>
       </c>
-      <c r="D23" t="inlineStr"/>
+      <c r="D23" t="n">
+        <v>0.9938782085461598</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -724,7 +768,9 @@
       <c r="C24" t="n">
         <v>32.62033579304236</v>
       </c>
-      <c r="D24" t="inlineStr"/>
+      <c r="D24" t="n">
+        <v>0.9959686255842534</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -736,7 +782,9 @@
       <c r="C25" t="n">
         <v>66.86694939091855</v>
       </c>
-      <c r="D25" t="inlineStr"/>
+      <c r="D25" t="n">
+        <v>0.9901155643413012</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -748,7 +796,9 @@
       <c r="C26" t="n">
         <v>61.39125059256289</v>
       </c>
-      <c r="D26" t="inlineStr"/>
+      <c r="D26" t="n">
+        <v>0.9940293171138485</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -760,7 +810,9 @@
       <c r="C27" t="n">
         <v>27.60097501061821</v>
       </c>
-      <c r="D27" t="inlineStr"/>
+      <c r="D27" t="n">
+        <v>0.9932866272101916</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -772,7 +824,9 @@
       <c r="C28" t="n">
         <v>57.44548841854294</v>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="n">
+        <v>0.991758578398844</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -784,7 +838,9 @@
       <c r="C29" t="n">
         <v>64.2897180394438</v>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="D29" t="n">
+        <v>0.9953537928390545</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -796,7 +852,9 @@
       <c r="C30" t="n">
         <v>51.04424473508528</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="D30" t="n">
+        <v>0.9939178184035558</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -808,7 +866,9 @@
       <c r="C31" t="n">
         <v>26.35625682329916</v>
       </c>
-      <c r="D31" t="inlineStr"/>
+      <c r="D31" t="n">
+        <v>0.9926999235337064</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -820,7 +880,9 @@
       <c r="C32" t="n">
         <v>47.49475732167166</v>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="D32" t="n">
+        <v>0.991884745091126</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -832,7 +894,9 @@
       <c r="C33" t="n">
         <v>37.53758065048235</v>
       </c>
-      <c r="D33" t="inlineStr"/>
+      <c r="D33" t="n">
+        <v>0.9978716165147297</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -844,7 +908,9 @@
       <c r="C34" t="n">
         <v>37.42441453674519</v>
       </c>
-      <c r="D34" t="inlineStr"/>
+      <c r="D34" t="n">
+        <v>0.9971771608396929</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -856,7 +922,9 @@
       <c r="C35" t="n">
         <v>54.82631099740421</v>
       </c>
-      <c r="D35" t="inlineStr"/>
+      <c r="D35" t="n">
+        <v>0.9954603870901648</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -868,7 +936,9 @@
       <c r="C36" t="n">
         <v>52.8998657286197</v>
       </c>
-      <c r="D36" t="inlineStr"/>
+      <c r="D36" t="n">
+        <v>0.9931059052080056</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -880,7 +950,9 @@
       <c r="C37" t="n">
         <v>64.07692484117138</v>
       </c>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="n">
+        <v>0.9985213781188168</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -892,7 +964,9 @@
       <c r="C38" t="n">
         <v>15.02018996783411</v>
       </c>
-      <c r="D38" t="inlineStr"/>
+      <c r="D38" t="n">
+        <v>0.9950703963705229</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -904,7 +978,9 @@
       <c r="C39" t="n">
         <v>23.07587490327965</v>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="D39" t="n">
+        <v>0.9938948646565796</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -916,7 +992,9 @@
       <c r="C40" t="n">
         <v>58.40841188526452</v>
       </c>
-      <c r="D40" t="inlineStr"/>
+      <c r="D40" t="n">
+        <v>0.998104046391038</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -928,7 +1006,9 @@
       <c r="C41" t="n">
         <v>31.82746499262569</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="D41" t="n">
+        <v>0.9928740762351168</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -940,7 +1020,9 @@
       <c r="C42" t="n">
         <v>35.37733090673469</v>
       </c>
-      <c r="D42" t="inlineStr"/>
+      <c r="D42" t="n">
+        <v>0.996263953831204</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -952,7 +1034,9 @@
       <c r="C43" t="n">
         <v>41.61615719019</v>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="n">
+        <v>0.9928243829453614</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -964,7 +1048,9 @@
       <c r="C44" t="n">
         <v>44.81145220748102</v>
       </c>
-      <c r="D44" t="inlineStr"/>
+      <c r="D44" t="n">
+        <v>0.9923539774168062</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -976,7 +1062,9 @@
       <c r="C45" t="n">
         <v>49.06743572749054</v>
       </c>
-      <c r="D45" t="inlineStr"/>
+      <c r="D45" t="n">
+        <v>0.9963075680055077</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -988,7 +1076,9 @@
       <c r="C46" t="n">
         <v>33.5774453963048</v>
       </c>
-      <c r="D46" t="inlineStr"/>
+      <c r="D46" t="n">
+        <v>0.9920510278101662</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1000,7 +1090,9 @@
       <c r="C47" t="n">
         <v>57.46522201167969</v>
       </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="n">
+        <v>0.994437992906864</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1012,7 +1104,9 @@
       <c r="C48" t="n">
         <v>52.03102919872997</v>
       </c>
-      <c r="D48" t="inlineStr"/>
+      <c r="D48" t="n">
+        <v>0.995220256077185</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1024,7 +1118,9 @@
       <c r="C49" t="n">
         <v>50.57254956738563</v>
       </c>
-      <c r="D49" t="inlineStr"/>
+      <c r="D49" t="n">
+        <v>0.9917001572827902</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1036,7 +1132,9 @@
       <c r="C50" t="n">
         <v>48.54148684428007</v>
       </c>
-      <c r="D50" t="inlineStr"/>
+      <c r="D50" t="n">
+        <v>0.9965811659252261</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1048,7 +1146,9 @@
       <c r="C51" t="n">
         <v>73.82498461236125</v>
       </c>
-      <c r="D51" t="inlineStr"/>
+      <c r="D51" t="n">
+        <v>0.9949363475816216</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1060,7 +1160,9 @@
       <c r="C52" t="n">
         <v>64.0560547756331</v>
       </c>
-      <c r="D52" t="inlineStr"/>
+      <c r="D52" t="n">
+        <v>0.9955935293366335</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1072,7 +1174,9 @@
       <c r="C53" t="n">
         <v>44.29222473466736</v>
       </c>
-      <c r="D53" t="inlineStr"/>
+      <c r="D53" t="n">
+        <v>0.9933492988511715</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1084,7 +1188,9 @@
       <c r="C54" t="n">
         <v>59.51537785616269</v>
       </c>
-      <c r="D54" t="inlineStr"/>
+      <c r="D54" t="n">
+        <v>0.9937817393392857</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1096,7 +1202,9 @@
       <c r="C55" t="n">
         <v>55.06770176992225</v>
       </c>
-      <c r="D55" t="inlineStr"/>
+      <c r="D55" t="n">
+        <v>0.9944534671012535</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1108,7 +1216,9 @@
       <c r="C56" t="n">
         <v>51.2529958529192</v>
       </c>
-      <c r="D56" t="inlineStr"/>
+      <c r="D56" t="n">
+        <v>0.9942297382116555</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1120,7 +1230,9 @@
       <c r="C57" t="n">
         <v>32.35552130588029</v>
       </c>
-      <c r="D57" t="inlineStr"/>
+      <c r="D57" t="n">
+        <v>0.9960807530056466</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1132,7 +1244,9 @@
       <c r="C58" t="n">
         <v>52.65079504580522</v>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="n">
+        <v>0.9951945975404658</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1144,7 +1258,9 @@
       <c r="C59" t="n">
         <v>53.2344844792981</v>
       </c>
-      <c r="D59" t="inlineStr"/>
+      <c r="D59" t="n">
+        <v>0.9937464357869322</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1156,7 +1272,9 @@
       <c r="C60" t="n">
         <v>55.85981383545153</v>
       </c>
-      <c r="D60" t="inlineStr"/>
+      <c r="D60" t="n">
+        <v>0.9900162211824614</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1168,7 +1286,9 @@
       <c r="C61" t="n">
         <v>56.84249730850535</v>
       </c>
-      <c r="D61" t="inlineStr"/>
+      <c r="D61" t="n">
+        <v>0.9971462795469795</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1180,7 +1300,9 @@
       <c r="C62" t="n">
         <v>56.04683541536205</v>
       </c>
-      <c r="D62" t="inlineStr"/>
+      <c r="D62" t="n">
+        <v>0.994674457990299</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1192,7 +1314,9 @@
       <c r="C63" t="n">
         <v>42.9238407328732</v>
       </c>
-      <c r="D63" t="inlineStr"/>
+      <c r="D63" t="n">
+        <v>0.9929389019743015</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1204,7 +1328,9 @@
       <c r="C64" t="n">
         <v>67.33541070056265</v>
       </c>
-      <c r="D64" t="inlineStr"/>
+      <c r="D64" t="n">
+        <v>0.9944995952017007</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1216,7 +1342,9 @@
       <c r="C65" t="n">
         <v>46.42083313914934</v>
       </c>
-      <c r="D65" t="inlineStr"/>
+      <c r="D65" t="n">
+        <v>0.9908410134014516</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1228,7 +1356,9 @@
       <c r="C66" t="n">
         <v>20.15246335861512</v>
       </c>
-      <c r="D66" t="inlineStr"/>
+      <c r="D66" t="n">
+        <v>0.9981423366529801</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1240,7 +1370,9 @@
       <c r="C67" t="n">
         <v>64.71781357938394</v>
       </c>
-      <c r="D67" t="inlineStr"/>
+      <c r="D67" t="n">
+        <v>0.9989076255082605</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1252,7 +1384,9 @@
       <c r="C68" t="n">
         <v>20.9709849543949</v>
       </c>
-      <c r="D68" t="inlineStr"/>
+      <c r="D68" t="n">
+        <v>0.9905286169576403</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -1264,7 +1398,9 @@
       <c r="C69" t="n">
         <v>54.59209029064667</v>
       </c>
-      <c r="D69" t="inlineStr"/>
+      <c r="D69" t="n">
+        <v>0.9932240809673224</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1276,7 +1412,9 @@
       <c r="C70" t="n">
         <v>54.35771212243785</v>
       </c>
-      <c r="D70" t="inlineStr"/>
+      <c r="D70" t="n">
+        <v>0.9965705812003718</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -1288,7 +1426,9 @@
       <c r="C71" t="n">
         <v>55.59379252137557</v>
       </c>
-      <c r="D71" t="inlineStr"/>
+      <c r="D71" t="n">
+        <v>0.9928281431809609</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -1300,7 +1440,9 @@
       <c r="C72" t="n">
         <v>66.00212359285925</v>
       </c>
-      <c r="D72" t="inlineStr"/>
+      <c r="D72" t="n">
+        <v>0.99510344782528</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -1312,7 +1454,9 @@
       <c r="C73" t="n">
         <v>50.87657503292501</v>
       </c>
-      <c r="D73" t="inlineStr"/>
+      <c r="D73" t="n">
+        <v>0.9937491386608353</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1324,7 +1468,9 @@
       <c r="C74" t="n">
         <v>40.3001338986972</v>
       </c>
-      <c r="D74" t="inlineStr"/>
+      <c r="D74" t="n">
+        <v>0.9969679094186779</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -1336,7 +1482,9 @@
       <c r="C75" t="n">
         <v>43.29408133550469</v>
       </c>
-      <c r="D75" t="inlineStr"/>
+      <c r="D75" t="n">
+        <v>0.9986261796086763</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1348,7 +1496,9 @@
       <c r="C76" t="n">
         <v>72.45615876012165</v>
       </c>
-      <c r="D76" t="inlineStr"/>
+      <c r="D76" t="n">
+        <v>0.9979955588368501</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -1360,7 +1510,9 @@
       <c r="C77" t="n">
         <v>71.96958543119473</v>
       </c>
-      <c r="D77" t="inlineStr"/>
+      <c r="D77" t="n">
+        <v>0.9955884191868004</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -1372,7 +1524,9 @@
       <c r="C78" t="n">
         <v>31.71903097672782</v>
       </c>
-      <c r="D78" t="inlineStr"/>
+      <c r="D78" t="n">
+        <v>0.9914424688140127</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -1384,7 +1538,9 @@
       <c r="C79" t="n">
         <v>24.78238876433949</v>
       </c>
-      <c r="D79" t="inlineStr"/>
+      <c r="D79" t="n">
+        <v>0.9985235587498049</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1396,7 +1552,9 @@
       <c r="C80" t="n">
         <v>35.78474079132059</v>
       </c>
-      <c r="D80" t="inlineStr"/>
+      <c r="D80" t="n">
+        <v>0.9902126918580459</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1408,7 +1566,9 @@
       <c r="C81" t="n">
         <v>85.86880632972213</v>
       </c>
-      <c r="D81" t="inlineStr"/>
+      <c r="D81" t="n">
+        <v>0.9926793851077877</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -1420,7 +1580,9 @@
       <c r="C82" t="n">
         <v>54.84551943934476</v>
       </c>
-      <c r="D82" t="inlineStr"/>
+      <c r="D82" t="n">
+        <v>0.9925345214379053</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -1432,7 +1594,9 @@
       <c r="C83" t="n">
         <v>42.02852297835588</v>
       </c>
-      <c r="D83" t="inlineStr"/>
+      <c r="D83" t="n">
+        <v>0.9960464338355043</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -1444,7 +1608,9 @@
       <c r="C84" t="n">
         <v>21.24799500474111</v>
       </c>
-      <c r="D84" t="inlineStr"/>
+      <c r="D84" t="n">
+        <v>0.9943862675946527</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -1456,7 +1622,9 @@
       <c r="C85" t="n">
         <v>29.26763733809423</v>
       </c>
-      <c r="D85" t="inlineStr"/>
+      <c r="D85" t="n">
+        <v>0.990835996938817</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1468,7 +1636,9 @@
       <c r="C86" t="n">
         <v>26.00454916311631</v>
       </c>
-      <c r="D86" t="inlineStr"/>
+      <c r="D86" t="n">
+        <v>0.9901157209897044</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -1480,7 +1650,9 @@
       <c r="C87" t="n">
         <v>49.24023764655826</v>
       </c>
-      <c r="D87" t="inlineStr"/>
+      <c r="D87" t="n">
+        <v>0.9954388417209628</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -1492,7 +1664,9 @@
       <c r="C88" t="n">
         <v>58.69657861547959</v>
       </c>
-      <c r="D88" t="inlineStr"/>
+      <c r="D88" t="n">
+        <v>0.9944233499910683</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -1504,7 +1678,9 @@
       <c r="C89" t="n">
         <v>38.56371252741226</v>
       </c>
-      <c r="D89" t="inlineStr"/>
+      <c r="D89" t="n">
+        <v>0.9954124390920636</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -1516,7 +1692,9 @@
       <c r="C90" t="n">
         <v>52.50241733428958</v>
       </c>
-      <c r="D90" t="inlineStr"/>
+      <c r="D90" t="n">
+        <v>0.9950762147747898</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -1528,7 +1706,9 @@
       <c r="C91" t="n">
         <v>36.73129929489149</v>
       </c>
-      <c r="D91" t="inlineStr"/>
+      <c r="D91" t="n">
+        <v>0.9980141319746971</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -1540,7 +1720,9 @@
       <c r="C92" t="n">
         <v>38.354514288082</v>
       </c>
-      <c r="D92" t="inlineStr"/>
+      <c r="D92" t="n">
+        <v>0.9982655717208354</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -1552,7 +1734,9 @@
       <c r="C93" t="n">
         <v>35.67810581622993</v>
       </c>
-      <c r="D93" t="inlineStr"/>
+      <c r="D93" t="n">
+        <v>0.9916943144499213</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -1564,7 +1748,9 @@
       <c r="C94" t="n">
         <v>53.07213893313723</v>
       </c>
-      <c r="D94" t="inlineStr"/>
+      <c r="D94" t="n">
+        <v>0.9984790878252348</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1576,7 +1762,9 @@
       <c r="C95" t="n">
         <v>48.86920189220226</v>
       </c>
-      <c r="D95" t="inlineStr"/>
+      <c r="D95" t="n">
+        <v>0.9970895396369051</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -1588,7 +1776,9 @@
       <c r="C96" t="n">
         <v>62.85358877955228</v>
       </c>
-      <c r="D96" t="inlineStr"/>
+      <c r="D96" t="n">
+        <v>0.9957512362700067</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -1600,7 +1790,9 @@
       <c r="C97" t="n">
         <v>51.47706433991497</v>
       </c>
-      <c r="D97" t="inlineStr"/>
+      <c r="D97" t="n">
+        <v>0.9959364654074185</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -1612,7 +1804,9 @@
       <c r="C98" t="n">
         <v>62.72713000736199</v>
       </c>
-      <c r="D98" t="inlineStr"/>
+      <c r="D98" t="n">
+        <v>0.9949145420691058</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -1624,7 +1818,9 @@
       <c r="C99" t="n">
         <v>30.1299770846383</v>
       </c>
-      <c r="D99" t="inlineStr"/>
+      <c r="D99" t="n">
+        <v>0.9982553696967855</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -1636,7 +1832,9 @@
       <c r="C100" t="n">
         <v>36.75800440157938</v>
       </c>
-      <c r="D100" t="inlineStr"/>
+      <c r="D100" t="n">
+        <v>0.9920993688558012</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -1648,7 +1846,9 @@
       <c r="C101" t="n">
         <v>63.89390408530792</v>
       </c>
-      <c r="D101" t="inlineStr"/>
+      <c r="D101" t="n">
+        <v>0.9953938439304262</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -1660,7 +1860,9 @@
       <c r="C102" t="n">
         <v>26.79910170703495</v>
       </c>
-      <c r="D102" t="inlineStr"/>
+      <c r="D102" t="n">
+        <v>0.9973281875568448</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -1672,7 +1874,9 @@
       <c r="C103" t="n">
         <v>60.78466344124584</v>
       </c>
-      <c r="D103" t="inlineStr"/>
+      <c r="D103" t="n">
+        <v>0.9912128530645902</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -1684,7 +1888,9 @@
       <c r="C104" t="n">
         <v>50.48567520359704</v>
       </c>
-      <c r="D104" t="inlineStr"/>
+      <c r="D104" t="n">
+        <v>0.9955395744692298</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -1696,7 +1902,9 @@
       <c r="C105" t="n">
         <v>41.35935978814719</v>
       </c>
-      <c r="D105" t="inlineStr"/>
+      <c r="D105" t="n">
+        <v>0.9936255012797661</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -1708,7 +1916,9 @@
       <c r="C106" t="n">
         <v>42.82388935866014</v>
       </c>
-      <c r="D106" t="inlineStr"/>
+      <c r="D106" t="n">
+        <v>0.9968943270731966</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -1720,7 +1930,9 @@
       <c r="C107" t="n">
         <v>68.23917794835043</v>
       </c>
-      <c r="D107" t="inlineStr"/>
+      <c r="D107" t="n">
+        <v>0.9906094292455848</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -1732,7 +1944,9 @@
       <c r="C108" t="n">
         <v>59.83732978424243</v>
       </c>
-      <c r="D108" t="inlineStr"/>
+      <c r="D108" t="n">
+        <v>0.9954613294293079</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -1744,7 +1958,9 @@
       <c r="C109" t="n">
         <v>74.63434472715409</v>
       </c>
-      <c r="D109" t="inlineStr"/>
+      <c r="D109" t="n">
+        <v>0.9977137082098798</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -1756,7 +1972,9 @@
       <c r="C110" t="n">
         <v>43.8272972250524</v>
       </c>
-      <c r="D110" t="inlineStr"/>
+      <c r="D110" t="n">
+        <v>0.9956551307612678</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -1768,7 +1986,9 @@
       <c r="C111" t="n">
         <v>38.43265364638556</v>
       </c>
-      <c r="D111" t="inlineStr"/>
+      <c r="D111" t="n">
+        <v>0.9928920392590816</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -1780,7 +2000,9 @@
       <c r="C112" t="n">
         <v>43.35818692272822</v>
       </c>
-      <c r="D112" t="inlineStr"/>
+      <c r="D112" t="n">
+        <v>0.995902164503297</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -1792,7 +2014,9 @@
       <c r="C113" t="n">
         <v>38.24494164978585</v>
       </c>
-      <c r="D113" t="inlineStr"/>
+      <c r="D113" t="n">
+        <v>0.9930433755846241</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -1804,7 +2028,9 @@
       <c r="C114" t="n">
         <v>63.72798095751364</v>
       </c>
-      <c r="D114" t="inlineStr"/>
+      <c r="D114" t="n">
+        <v>0.9960173350956908</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -1816,7 +2042,9 @@
       <c r="C115" t="n">
         <v>67.53649305633806</v>
       </c>
-      <c r="D115" t="inlineStr"/>
+      <c r="D115" t="n">
+        <v>0.9911550996129784</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -1828,7 +2056,9 @@
       <c r="C116" t="n">
         <v>32.72351644182054</v>
       </c>
-      <c r="D116" t="inlineStr"/>
+      <c r="D116" t="n">
+        <v>0.992519925697763</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -1840,7 +2070,9 @@
       <c r="C117" t="n">
         <v>61.59257328408566</v>
       </c>
-      <c r="D117" t="inlineStr"/>
+      <c r="D117" t="n">
+        <v>0.9902944654037722</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -1852,7 +2084,9 @@
       <c r="C118" t="n">
         <v>25.38818198523678</v>
       </c>
-      <c r="D118" t="inlineStr"/>
+      <c r="D118" t="n">
+        <v>0.9907551845006642</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -1864,7 +2098,9 @@
       <c r="C119" t="n">
         <v>45.79677033582375</v>
       </c>
-      <c r="D119" t="inlineStr"/>
+      <c r="D119" t="n">
+        <v>0.9949929265783486</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -1876,7 +2112,9 @@
       <c r="C120" t="n">
         <v>37.48719016337304</v>
       </c>
-      <c r="D120" t="inlineStr"/>
+      <c r="D120" t="n">
+        <v>0.9920852839925307</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -1888,7 +2126,9 @@
       <c r="C121" t="n">
         <v>32.63044854100505</v>
       </c>
-      <c r="D121" t="inlineStr"/>
+      <c r="D121" t="n">
+        <v>0.9946447432887395</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -1900,7 +2140,9 @@
       <c r="C122" t="n">
         <v>68.28707584039341</v>
       </c>
-      <c r="D122" t="inlineStr"/>
+      <c r="D122" t="n">
+        <v>0.9959361257976556</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -1912,7 +2154,9 @@
       <c r="C123" t="n">
         <v>33.24305624591818</v>
       </c>
-      <c r="D123" t="inlineStr"/>
+      <c r="D123" t="n">
+        <v>0.9979306756141457</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -1924,7 +2168,9 @@
       <c r="C124" t="n">
         <v>44.03556352239427</v>
       </c>
-      <c r="D124" t="inlineStr"/>
+      <c r="D124" t="n">
+        <v>0.9931955491312968</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -1936,7 +2182,9 @@
       <c r="C125" t="n">
         <v>42.74363943603997</v>
       </c>
-      <c r="D125" t="inlineStr"/>
+      <c r="D125" t="n">
+        <v>0.9928681106979487</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -1948,7 +2196,9 @@
       <c r="C126" t="n">
         <v>58.85095317494391</v>
       </c>
-      <c r="D126" t="inlineStr"/>
+      <c r="D126" t="n">
+        <v>0.9928230006740743</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -1960,7 +2210,9 @@
       <c r="C127" t="n">
         <v>16.17394847958799</v>
       </c>
-      <c r="D127" t="inlineStr"/>
+      <c r="D127" t="n">
+        <v>0.9910606468007196</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -1972,7 +2224,9 @@
       <c r="C128" t="n">
         <v>33.87766682607845</v>
       </c>
-      <c r="D128" t="inlineStr"/>
+      <c r="D128" t="n">
+        <v>0.9959686502819154</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -1984,7 +2238,9 @@
       <c r="C129" t="n">
         <v>47.00209216877489</v>
       </c>
-      <c r="D129" t="inlineStr"/>
+      <c r="D129" t="n">
+        <v>0.9973768912329349</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -1996,7 +2252,9 @@
       <c r="C130" t="n">
         <v>21.82843164035993</v>
       </c>
-      <c r="D130" t="inlineStr"/>
+      <c r="D130" t="n">
+        <v>0.9942570437477669</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -2008,7 +2266,9 @@
       <c r="C131" t="n">
         <v>60.99389115413728</v>
       </c>
-      <c r="D131" t="inlineStr"/>
+      <c r="D131" t="n">
+        <v>0.9950246765725369</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -2020,7 +2280,9 @@
       <c r="C132" t="n">
         <v>56.44673584598896</v>
       </c>
-      <c r="D132" t="inlineStr"/>
+      <c r="D132" t="n">
+        <v>0.9986263210232605</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -2032,7 +2294,9 @@
       <c r="C133" t="n">
         <v>69.7668412155984</v>
       </c>
-      <c r="D133" t="inlineStr"/>
+      <c r="D133" t="n">
+        <v>0.9962902365448724</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2044,7 +2308,9 @@
       <c r="C134" t="n">
         <v>61.90100495581607</v>
       </c>
-      <c r="D134" t="inlineStr"/>
+      <c r="D134" t="n">
+        <v>0.9967053139798289</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -2056,7 +2322,9 @@
       <c r="C135" t="n">
         <v>67.47581972462075</v>
       </c>
-      <c r="D135" t="inlineStr"/>
+      <c r="D135" t="n">
+        <v>0.9980054852157407</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -2068,7 +2336,9 @@
       <c r="C136" t="n">
         <v>56.0214981912111</v>
       </c>
-      <c r="D136" t="inlineStr"/>
+      <c r="D136" t="n">
+        <v>0.9919421151847571</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2080,7 +2350,9 @@
       <c r="C137" t="n">
         <v>50.95247214583335</v>
       </c>
-      <c r="D137" t="inlineStr"/>
+      <c r="D137" t="n">
+        <v>0.9958514945248862</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2092,7 +2364,9 @@
       <c r="C138" t="n">
         <v>53.57551639207747</v>
       </c>
-      <c r="D138" t="inlineStr"/>
+      <c r="D138" t="n">
+        <v>0.9964565505479376</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2104,7 +2378,9 @@
       <c r="C139" t="n">
         <v>50.14878729140165</v>
       </c>
-      <c r="D139" t="inlineStr"/>
+      <c r="D139" t="n">
+        <v>0.9975800513675117</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -2116,7 +2392,9 @@
       <c r="C140" t="n">
         <v>39.11919311989337</v>
       </c>
-      <c r="D140" t="inlineStr"/>
+      <c r="D140" t="n">
+        <v>0.9930940699140171</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -2128,7 +2406,9 @@
       <c r="C141" t="n">
         <v>57.67393992818478</v>
       </c>
-      <c r="D141" t="inlineStr"/>
+      <c r="D141" t="n">
+        <v>0.9961991523514174</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -2140,7 +2420,9 @@
       <c r="C142" t="n">
         <v>59.98976470976152</v>
       </c>
-      <c r="D142" t="inlineStr"/>
+      <c r="D142" t="n">
+        <v>0.9954396054522234</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -2152,7 +2434,9 @@
       <c r="C143" t="n">
         <v>61.29403023760543</v>
       </c>
-      <c r="D143" t="inlineStr"/>
+      <c r="D143" t="n">
+        <v>0.993684249304404</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -2164,7 +2448,9 @@
       <c r="C144" t="n">
         <v>41.06339365608342</v>
       </c>
-      <c r="D144" t="inlineStr"/>
+      <c r="D144" t="n">
+        <v>0.9909151718137394</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -2176,7 +2462,9 @@
       <c r="C145" t="n">
         <v>71.71488219151669</v>
       </c>
-      <c r="D145" t="inlineStr"/>
+      <c r="D145" t="n">
+        <v>0.9931774359040483</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -2188,7 +2476,9 @@
       <c r="C146" t="n">
         <v>33.21788065693907</v>
       </c>
-      <c r="D146" t="inlineStr"/>
+      <c r="D146" t="n">
+        <v>0.9986713627330843</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -2200,7 +2490,9 @@
       <c r="C147" t="n">
         <v>35.76532379625473</v>
       </c>
-      <c r="D147" t="inlineStr"/>
+      <c r="D147" t="n">
+        <v>0.9919487115145151</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2212,7 +2504,9 @@
       <c r="C148" t="n">
         <v>50.30715431918719</v>
       </c>
-      <c r="D148" t="inlineStr"/>
+      <c r="D148" t="n">
+        <v>0.9910227419422936</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2224,7 +2518,9 @@
       <c r="C149" t="n">
         <v>41.70098183161208</v>
       </c>
-      <c r="D149" t="inlineStr"/>
+      <c r="D149" t="n">
+        <v>0.9933091148226331</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -2236,7 +2532,9 @@
       <c r="C150" t="n">
         <v>25.71370826456232</v>
       </c>
-      <c r="D150" t="inlineStr"/>
+      <c r="D150" t="n">
+        <v>0.9909088271289538</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -2248,7 +2546,9 @@
       <c r="C151" t="n">
         <v>26.49052869939182</v>
       </c>
-      <c r="D151" t="inlineStr"/>
+      <c r="D151" t="n">
+        <v>0.9924047903865264</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -2260,7 +2560,9 @@
       <c r="C152" t="n">
         <v>63.90692432390129</v>
       </c>
-      <c r="D152" t="inlineStr"/>
+      <c r="D152" t="n">
+        <v>0.9982301050989263</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -2272,7 +2574,9 @@
       <c r="C153" t="n">
         <v>63.37928648737845</v>
       </c>
-      <c r="D153" t="inlineStr"/>
+      <c r="D153" t="n">
+        <v>0.9928690387330102</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -2284,7 +2588,9 @@
       <c r="C154" t="n">
         <v>25.12029222292051</v>
       </c>
-      <c r="D154" t="inlineStr"/>
+      <c r="D154" t="n">
+        <v>0.9952730056309215</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -2296,7 +2602,9 @@
       <c r="C155" t="n">
         <v>39.60329258760133</v>
       </c>
-      <c r="D155" t="inlineStr"/>
+      <c r="D155" t="n">
+        <v>0.9921487030159946</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -2308,7 +2616,9 @@
       <c r="C156" t="n">
         <v>12.21263075110782</v>
       </c>
-      <c r="D156" t="inlineStr"/>
+      <c r="D156" t="n">
+        <v>0.9960118193195865</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2320,7 +2630,9 @@
       <c r="C157" t="n">
         <v>30.54834043508056</v>
       </c>
-      <c r="D157" t="inlineStr"/>
+      <c r="D157" t="n">
+        <v>0.991148907488984</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2332,7 +2644,9 @@
       <c r="C158" t="n">
         <v>50.03149339688316</v>
       </c>
-      <c r="D158" t="inlineStr"/>
+      <c r="D158" t="n">
+        <v>0.9971082844494795</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -2344,7 +2658,9 @@
       <c r="C159" t="n">
         <v>47.94394853399143</v>
       </c>
-      <c r="D159" t="inlineStr"/>
+      <c r="D159" t="n">
+        <v>0.9938065144029443</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -2356,7 +2672,9 @@
       <c r="C160" t="n">
         <v>69.92956674357832</v>
       </c>
-      <c r="D160" t="inlineStr"/>
+      <c r="D160" t="n">
+        <v>0.9916529434838228</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -2368,7 +2686,9 @@
       <c r="C161" t="n">
         <v>31.9704602093228</v>
       </c>
-      <c r="D161" t="inlineStr"/>
+      <c r="D161" t="n">
+        <v>0.9968242460908364</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -2380,7 +2700,9 @@
       <c r="C162" t="n">
         <v>38.96577069630239</v>
       </c>
-      <c r="D162" t="inlineStr"/>
+      <c r="D162" t="n">
+        <v>0.9949885428512451</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -2392,7 +2714,9 @@
       <c r="C163" t="n">
         <v>39.39751136993004</v>
       </c>
-      <c r="D163" t="inlineStr"/>
+      <c r="D163" t="n">
+        <v>0.9939433050929787</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -2404,7 +2728,9 @@
       <c r="C164" t="n">
         <v>70.84264618277928</v>
       </c>
-      <c r="D164" t="inlineStr"/>
+      <c r="D164" t="n">
+        <v>0.992165634376324</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -2416,7 +2742,9 @@
       <c r="C165" t="n">
         <v>33.99966038162763</v>
       </c>
-      <c r="D165" t="inlineStr"/>
+      <c r="D165" t="n">
+        <v>0.9970322930387524</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -2428,7 +2756,9 @@
       <c r="C166" t="n">
         <v>56.52139609313584</v>
       </c>
-      <c r="D166" t="inlineStr"/>
+      <c r="D166" t="n">
+        <v>0.9932875655103311</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -2440,7 +2770,9 @@
       <c r="C167" t="n">
         <v>51.63354419283532</v>
       </c>
-      <c r="D167" t="inlineStr"/>
+      <c r="D167" t="n">
+        <v>0.9903878162157114</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -2452,7 +2784,9 @@
       <c r="C168" t="n">
         <v>47.10708506835977</v>
       </c>
-      <c r="D168" t="inlineStr"/>
+      <c r="D168" t="n">
+        <v>0.9986883234286021</v>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -2464,7 +2798,9 @@
       <c r="C169" t="n">
         <v>55.25408342657246</v>
       </c>
-      <c r="D169" t="inlineStr"/>
+      <c r="D169" t="n">
+        <v>0.990274183273124</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -2476,7 +2812,9 @@
       <c r="C170" t="n">
         <v>60.65846113009473</v>
       </c>
-      <c r="D170" t="inlineStr"/>
+      <c r="D170" t="n">
+        <v>0.9910842216986149</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -2488,7 +2826,9 @@
       <c r="C171" t="n">
         <v>89.11758782502773</v>
       </c>
-      <c r="D171" t="inlineStr"/>
+      <c r="D171" t="n">
+        <v>0.9941923127789584</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -2500,7 +2840,9 @@
       <c r="C172" t="n">
         <v>34.15141111167516</v>
       </c>
-      <c r="D172" t="inlineStr"/>
+      <c r="D172" t="n">
+        <v>0.9918706944741474</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -2512,7 +2854,9 @@
       <c r="C173" t="n">
         <v>81.70343159249632</v>
       </c>
-      <c r="D173" t="inlineStr"/>
+      <c r="D173" t="n">
+        <v>0.9930162153382749</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -2524,7 +2868,9 @@
       <c r="C174" t="n">
         <v>66.67672188427332</v>
       </c>
-      <c r="D174" t="inlineStr"/>
+      <c r="D174" t="n">
+        <v>0.9951080871774001</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -2536,7 +2882,9 @@
       <c r="C175" t="n">
         <v>55.87154050616485</v>
       </c>
-      <c r="D175" t="inlineStr"/>
+      <c r="D175" t="n">
+        <v>0.9986205775703306</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -2548,7 +2896,9 @@
       <c r="C176" t="n">
         <v>38.00322570895611</v>
       </c>
-      <c r="D176" t="inlineStr"/>
+      <c r="D176" t="n">
+        <v>0.9984268100183206</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -2560,7 +2910,9 @@
       <c r="C177" t="n">
         <v>29.69824828000953</v>
       </c>
-      <c r="D177" t="inlineStr"/>
+      <c r="D177" t="n">
+        <v>0.9906650637826071</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -2572,7 +2924,9 @@
       <c r="C178" t="n">
         <v>51.10642431092796</v>
       </c>
-      <c r="D178" t="inlineStr"/>
+      <c r="D178" t="n">
+        <v>0.9976798229063399</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -2584,7 +2938,9 @@
       <c r="C179" t="n">
         <v>58.24256654083357</v>
       </c>
-      <c r="D179" t="inlineStr"/>
+      <c r="D179" t="n">
+        <v>0.9915104128961902</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -2596,7 +2952,9 @@
       <c r="C180" t="n">
         <v>57.90753875284465</v>
       </c>
-      <c r="D180" t="inlineStr"/>
+      <c r="D180" t="n">
+        <v>0.9973028958525291</v>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -2608,7 +2966,9 @@
       <c r="C181" t="n">
         <v>37.82288482564915</v>
       </c>
-      <c r="D181" t="inlineStr"/>
+      <c r="D181" t="n">
+        <v>0.9926671249606338</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -2620,7 +2980,9 @@
       <c r="C182" t="n">
         <v>59.72710216882905</v>
       </c>
-      <c r="D182" t="inlineStr"/>
+      <c r="D182" t="n">
+        <v>0.9964605092155461</v>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -2632,7 +2994,9 @@
       <c r="C183" t="n">
         <v>30.0882005832016</v>
       </c>
-      <c r="D183" t="inlineStr"/>
+      <c r="D183" t="n">
+        <v>0.9964691388452478</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -2644,7 +3008,9 @@
       <c r="C184" t="n">
         <v>50.0340207885088</v>
       </c>
-      <c r="D184" t="inlineStr"/>
+      <c r="D184" t="n">
+        <v>0.9976549613378072</v>
+      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -2656,7 +3022,9 @@
       <c r="C185" t="n">
         <v>22.99356530034146</v>
       </c>
-      <c r="D185" t="inlineStr"/>
+      <c r="D185" t="n">
+        <v>0.9988166326396635</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -2668,7 +3036,9 @@
       <c r="C186" t="n">
         <v>70.53643160720347</v>
       </c>
-      <c r="D186" t="inlineStr"/>
+      <c r="D186" t="n">
+        <v>0.992479327675767</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -2680,7 +3050,9 @@
       <c r="C187" t="n">
         <v>69.30669020013021</v>
       </c>
-      <c r="D187" t="inlineStr"/>
+      <c r="D187" t="n">
+        <v>0.9956547761280695</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -2692,7 +3064,9 @@
       <c r="C188" t="n">
         <v>53.28708600267237</v>
       </c>
-      <c r="D188" t="inlineStr"/>
+      <c r="D188" t="n">
+        <v>0.9966533471607333</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" t="n">
@@ -2704,7 +3078,9 @@
       <c r="C189" t="n">
         <v>58.33525434379268</v>
       </c>
-      <c r="D189" t="inlineStr"/>
+      <c r="D189" t="n">
+        <v>0.9907166640381805</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -2716,7 +3092,9 @@
       <c r="C190" t="n">
         <v>52.21783588359124</v>
       </c>
-      <c r="D190" t="inlineStr"/>
+      <c r="D190" t="n">
+        <v>0.9959666520399196</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" t="n">
@@ -2728,7 +3106,9 @@
       <c r="C191" t="n">
         <v>73.04385275833977</v>
       </c>
-      <c r="D191" t="inlineStr"/>
+      <c r="D191" t="n">
+        <v>0.9928936396377742</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="n">
@@ -2740,7 +3120,9 @@
       <c r="C192" t="n">
         <v>47.88198415669979</v>
       </c>
-      <c r="D192" t="inlineStr"/>
+      <c r="D192" t="n">
+        <v>0.9914532213839485</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="n">
@@ -2752,7 +3134,9 @@
       <c r="C193" t="n">
         <v>31.82557362505747</v>
       </c>
-      <c r="D193" t="inlineStr"/>
+      <c r="D193" t="n">
+        <v>0.9949452440205129</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="n">
@@ -2764,7 +3148,9 @@
       <c r="C194" t="n">
         <v>7.703496491937528</v>
       </c>
-      <c r="D194" t="inlineStr"/>
+      <c r="D194" t="n">
+        <v>0.9941569523736981</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -2776,7 +3162,9 @@
       <c r="C195" t="n">
         <v>57.38510043723399</v>
       </c>
-      <c r="D195" t="inlineStr"/>
+      <c r="D195" t="n">
+        <v>0.9951937184966392</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" t="n">
@@ -2788,7 +3176,9 @@
       <c r="C196" t="n">
         <v>21.07210778365031</v>
       </c>
-      <c r="D196" t="inlineStr"/>
+      <c r="D196" t="n">
+        <v>0.9957772583136302</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" t="n">
@@ -2800,7 +3190,9 @@
       <c r="C197" t="n">
         <v>50.77438967751996</v>
       </c>
-      <c r="D197" t="inlineStr"/>
+      <c r="D197" t="n">
+        <v>0.9944880197521365</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" t="n">
@@ -2812,7 +3204,9 @@
       <c r="C198" t="n">
         <v>59.94433851813749</v>
       </c>
-      <c r="D198" t="inlineStr"/>
+      <c r="D198" t="n">
+        <v>0.9981463563669523</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" t="n">
@@ -2824,7 +3218,9 @@
       <c r="C199" t="n">
         <v>18.08351560802339</v>
       </c>
-      <c r="D199" t="inlineStr"/>
+      <c r="D199" t="n">
+        <v>0.9916012277855191</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="n">
@@ -2836,7 +3232,9 @@
       <c r="C200" t="n">
         <v>48.88290551241017</v>
       </c>
-      <c r="D200" t="inlineStr"/>
+      <c r="D200" t="n">
+        <v>0.9925991248410848</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -2848,7 +3246,9 @@
       <c r="C201" t="n">
         <v>60.19400006076078</v>
       </c>
-      <c r="D201" t="inlineStr"/>
+      <c r="D201" t="n">
+        <v>0.9932059947706208</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add four-tier spatial reliability PPO diagnostics
</commit_message>
<xml_diff>
--- a/data/task_parameters.xlsx
+++ b/data/task_parameters.xlsx
@@ -461,7 +461,7 @@
         <v>53.67919023703534</v>
       </c>
       <c r="D2" t="n">
-        <v>0.9916104133230789</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="3">
@@ -475,7 +475,7 @@
         <v>34.75107857408746</v>
       </c>
       <c r="D3" t="n">
-        <v>0.9957592184914363</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +489,7 @@
         <v>42.60628635542257</v>
       </c>
       <c r="D4" t="n">
-        <v>0.9942054156102914</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="5">
@@ -503,7 +503,7 @@
         <v>33.48190127293107</v>
       </c>
       <c r="D5" t="n">
-        <v>0.9933345047439724</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="6">
@@ -517,7 +517,7 @@
         <v>45.23196171646185</v>
       </c>
       <c r="D6" t="n">
-        <v>0.9931942560087869</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="7">
@@ -531,7 +531,7 @@
         <v>42.32918817317876</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9971146642126794</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="8">
@@ -545,7 +545,7 @@
         <v>44.44014536248625</v>
       </c>
       <c r="D8" t="n">
-        <v>0.9981462945300945</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="9">
@@ -559,7 +559,7 @@
         <v>47.94897151388241</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9915961787264075</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="10">
@@ -573,7 +573,7 @@
         <v>44.64165636479374</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9958750632241662</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="11">
@@ -587,7 +587,7 @@
         <v>28.02194103187311</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9926847249062001</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="12">
@@ -601,7 +601,7 @@
         <v>50.49475649543508</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9987026598014616</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="13">
@@ -615,7 +615,7 @@
         <v>40.71306000432234</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9982786514448355</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="14">
@@ -629,7 +629,7 @@
         <v>47.09592044693731</v>
       </c>
       <c r="D14" t="n">
-        <v>0.9957228372373018</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="15">
@@ -643,7 +643,7 @@
         <v>62.52548385599771</v>
       </c>
       <c r="D15" t="n">
-        <v>0.9967745888737117</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="16">
@@ -657,7 +657,7 @@
         <v>54.260886173613</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9946363832669012</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="17">
@@ -671,7 +671,7 @@
         <v>60.50559856437604</v>
       </c>
       <c r="D17" t="n">
-        <v>0.9974330573253801</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="18">
@@ -685,7 +685,7 @@
         <v>71.04614060419865</v>
       </c>
       <c r="D18" t="n">
-        <v>0.994035424908601</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="19">
@@ -699,7 +699,7 @@
         <v>58.55154095134137</v>
       </c>
       <c r="D19" t="n">
-        <v>0.9930493120798238</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="20">
@@ -713,7 +713,7 @@
         <v>51.66508863793452</v>
       </c>
       <c r="D20" t="n">
-        <v>0.9925010929395014</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="21">
@@ -727,7 +727,7 @@
         <v>78.40138622491851</v>
       </c>
       <c r="D21" t="n">
-        <v>0.9920369975115906</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="22">
@@ -741,7 +741,7 @@
         <v>48.7360258336366</v>
       </c>
       <c r="D22" t="n">
-        <v>0.9947323515901072</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="23">
@@ -755,7 +755,7 @@
         <v>49.85244703050946</v>
       </c>
       <c r="D23" t="n">
-        <v>0.9938782085461598</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="24">
@@ -769,7 +769,7 @@
         <v>32.62033579304236</v>
       </c>
       <c r="D24" t="n">
-        <v>0.9959686255842534</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="25">
@@ -783,7 +783,7 @@
         <v>66.86694939091855</v>
       </c>
       <c r="D25" t="n">
-        <v>0.9901155643413012</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="26">
@@ -797,7 +797,7 @@
         <v>61.39125059256289</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9940293171138485</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="27">
@@ -811,7 +811,7 @@
         <v>27.60097501061821</v>
       </c>
       <c r="D27" t="n">
-        <v>0.9932866272101916</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="28">
@@ -825,7 +825,7 @@
         <v>57.44548841854294</v>
       </c>
       <c r="D28" t="n">
-        <v>0.991758578398844</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="29">
@@ -839,7 +839,7 @@
         <v>64.2897180394438</v>
       </c>
       <c r="D29" t="n">
-        <v>0.9953537928390545</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="30">
@@ -853,7 +853,7 @@
         <v>51.04424473508528</v>
       </c>
       <c r="D30" t="n">
-        <v>0.9939178184035558</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="31">
@@ -867,7 +867,7 @@
         <v>26.35625682329916</v>
       </c>
       <c r="D31" t="n">
-        <v>0.9926999235337064</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="32">
@@ -881,7 +881,7 @@
         <v>47.49475732167166</v>
       </c>
       <c r="D32" t="n">
-        <v>0.991884745091126</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="33">
@@ -895,7 +895,7 @@
         <v>37.53758065048235</v>
       </c>
       <c r="D33" t="n">
-        <v>0.9978716165147297</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="34">
@@ -909,7 +909,7 @@
         <v>37.42441453674519</v>
       </c>
       <c r="D34" t="n">
-        <v>0.9971771608396929</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="35">
@@ -923,7 +923,7 @@
         <v>54.82631099740421</v>
       </c>
       <c r="D35" t="n">
-        <v>0.9954603870901648</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="36">
@@ -937,7 +937,7 @@
         <v>52.8998657286197</v>
       </c>
       <c r="D36" t="n">
-        <v>0.9931059052080056</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="37">
@@ -951,7 +951,7 @@
         <v>64.07692484117138</v>
       </c>
       <c r="D37" t="n">
-        <v>0.9985213781188168</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="38">
@@ -965,7 +965,7 @@
         <v>15.02018996783411</v>
       </c>
       <c r="D38" t="n">
-        <v>0.9950703963705229</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="39">
@@ -979,7 +979,7 @@
         <v>23.07587490327965</v>
       </c>
       <c r="D39" t="n">
-        <v>0.9938948646565796</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="40">
@@ -993,7 +993,7 @@
         <v>58.40841188526452</v>
       </c>
       <c r="D40" t="n">
-        <v>0.998104046391038</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="41">
@@ -1007,7 +1007,7 @@
         <v>31.82746499262569</v>
       </c>
       <c r="D41" t="n">
-        <v>0.9928740762351168</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="42">
@@ -1021,7 +1021,7 @@
         <v>35.37733090673469</v>
       </c>
       <c r="D42" t="n">
-        <v>0.996263953831204</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="43">
@@ -1035,7 +1035,7 @@
         <v>41.61615719019</v>
       </c>
       <c r="D43" t="n">
-        <v>0.9928243829453614</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="44">
@@ -1049,7 +1049,7 @@
         <v>44.81145220748102</v>
       </c>
       <c r="D44" t="n">
-        <v>0.9923539774168062</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="45">
@@ -1063,7 +1063,7 @@
         <v>49.06743572749054</v>
       </c>
       <c r="D45" t="n">
-        <v>0.9963075680055077</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="46">
@@ -1077,7 +1077,7 @@
         <v>33.5774453963048</v>
       </c>
       <c r="D46" t="n">
-        <v>0.9920510278101662</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="47">
@@ -1091,7 +1091,7 @@
         <v>57.46522201167969</v>
       </c>
       <c r="D47" t="n">
-        <v>0.994437992906864</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="48">
@@ -1105,7 +1105,7 @@
         <v>52.03102919872997</v>
       </c>
       <c r="D48" t="n">
-        <v>0.995220256077185</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="49">
@@ -1119,7 +1119,7 @@
         <v>50.57254956738563</v>
       </c>
       <c r="D49" t="n">
-        <v>0.9917001572827902</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="50">
@@ -1133,7 +1133,7 @@
         <v>48.54148684428007</v>
       </c>
       <c r="D50" t="n">
-        <v>0.9965811659252261</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="51">
@@ -1147,7 +1147,7 @@
         <v>73.82498461236125</v>
       </c>
       <c r="D51" t="n">
-        <v>0.9949363475816216</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="52">
@@ -1161,7 +1161,7 @@
         <v>64.0560547756331</v>
       </c>
       <c r="D52" t="n">
-        <v>0.9955935293366335</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="53">
@@ -1175,7 +1175,7 @@
         <v>44.29222473466736</v>
       </c>
       <c r="D53" t="n">
-        <v>0.9933492988511715</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="54">
@@ -1189,7 +1189,7 @@
         <v>59.51537785616269</v>
       </c>
       <c r="D54" t="n">
-        <v>0.9937817393392857</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="55">
@@ -1203,7 +1203,7 @@
         <v>55.06770176992225</v>
       </c>
       <c r="D55" t="n">
-        <v>0.9944534671012535</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="56">
@@ -1217,7 +1217,7 @@
         <v>51.2529958529192</v>
       </c>
       <c r="D56" t="n">
-        <v>0.9942297382116555</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="57">
@@ -1231,7 +1231,7 @@
         <v>32.35552130588029</v>
       </c>
       <c r="D57" t="n">
-        <v>0.9960807530056466</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="58">
@@ -1245,7 +1245,7 @@
         <v>52.65079504580522</v>
       </c>
       <c r="D58" t="n">
-        <v>0.9951945975404658</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="59">
@@ -1259,7 +1259,7 @@
         <v>53.2344844792981</v>
       </c>
       <c r="D59" t="n">
-        <v>0.9937464357869322</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="60">
@@ -1273,7 +1273,7 @@
         <v>55.85981383545153</v>
       </c>
       <c r="D60" t="n">
-        <v>0.9900162211824614</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="61">
@@ -1287,7 +1287,7 @@
         <v>56.84249730850535</v>
       </c>
       <c r="D61" t="n">
-        <v>0.9971462795469795</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="62">
@@ -1301,7 +1301,7 @@
         <v>56.04683541536205</v>
       </c>
       <c r="D62" t="n">
-        <v>0.994674457990299</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="63">
@@ -1315,7 +1315,7 @@
         <v>42.9238407328732</v>
       </c>
       <c r="D63" t="n">
-        <v>0.9929389019743015</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="64">
@@ -1329,7 +1329,7 @@
         <v>67.33541070056265</v>
       </c>
       <c r="D64" t="n">
-        <v>0.9944995952017007</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="65">
@@ -1343,7 +1343,7 @@
         <v>46.42083313914934</v>
       </c>
       <c r="D65" t="n">
-        <v>0.9908410134014516</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="66">
@@ -1357,7 +1357,7 @@
         <v>20.15246335861512</v>
       </c>
       <c r="D66" t="n">
-        <v>0.9981423366529801</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="67">
@@ -1371,7 +1371,7 @@
         <v>64.71781357938394</v>
       </c>
       <c r="D67" t="n">
-        <v>0.9989076255082605</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="68">
@@ -1385,7 +1385,7 @@
         <v>20.9709849543949</v>
       </c>
       <c r="D68" t="n">
-        <v>0.9905286169576403</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="69">
@@ -1399,7 +1399,7 @@
         <v>54.59209029064667</v>
       </c>
       <c r="D69" t="n">
-        <v>0.9932240809673224</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="70">
@@ -1413,7 +1413,7 @@
         <v>54.35771212243785</v>
       </c>
       <c r="D70" t="n">
-        <v>0.9965705812003718</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="71">
@@ -1427,7 +1427,7 @@
         <v>55.59379252137557</v>
       </c>
       <c r="D71" t="n">
-        <v>0.9928281431809609</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="72">
@@ -1441,7 +1441,7 @@
         <v>66.00212359285925</v>
       </c>
       <c r="D72" t="n">
-        <v>0.99510344782528</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="73">
@@ -1455,7 +1455,7 @@
         <v>50.87657503292501</v>
       </c>
       <c r="D73" t="n">
-        <v>0.9937491386608353</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="74">
@@ -1469,7 +1469,7 @@
         <v>40.3001338986972</v>
       </c>
       <c r="D74" t="n">
-        <v>0.9969679094186779</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="75">
@@ -1483,7 +1483,7 @@
         <v>43.29408133550469</v>
       </c>
       <c r="D75" t="n">
-        <v>0.9986261796086763</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="76">
@@ -1497,7 +1497,7 @@
         <v>72.45615876012165</v>
       </c>
       <c r="D76" t="n">
-        <v>0.9979955588368501</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="77">
@@ -1511,7 +1511,7 @@
         <v>71.96958543119473</v>
       </c>
       <c r="D77" t="n">
-        <v>0.9955884191868004</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="78">
@@ -1525,7 +1525,7 @@
         <v>31.71903097672782</v>
       </c>
       <c r="D78" t="n">
-        <v>0.9914424688140127</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="79">
@@ -1539,7 +1539,7 @@
         <v>24.78238876433949</v>
       </c>
       <c r="D79" t="n">
-        <v>0.9985235587498049</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="80">
@@ -1553,7 +1553,7 @@
         <v>35.78474079132059</v>
       </c>
       <c r="D80" t="n">
-        <v>0.9902126918580459</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="81">
@@ -1567,7 +1567,7 @@
         <v>85.86880632972213</v>
       </c>
       <c r="D81" t="n">
-        <v>0.9926793851077877</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="82">
@@ -1581,7 +1581,7 @@
         <v>54.84551943934476</v>
       </c>
       <c r="D82" t="n">
-        <v>0.9925345214379053</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="83">
@@ -1595,7 +1595,7 @@
         <v>42.02852297835588</v>
       </c>
       <c r="D83" t="n">
-        <v>0.9960464338355043</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="84">
@@ -1609,7 +1609,7 @@
         <v>21.24799500474111</v>
       </c>
       <c r="D84" t="n">
-        <v>0.9943862675946527</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="85">
@@ -1623,7 +1623,7 @@
         <v>29.26763733809423</v>
       </c>
       <c r="D85" t="n">
-        <v>0.990835996938817</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="86">
@@ -1637,7 +1637,7 @@
         <v>26.00454916311631</v>
       </c>
       <c r="D86" t="n">
-        <v>0.9901157209897044</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="87">
@@ -1651,7 +1651,7 @@
         <v>49.24023764655826</v>
       </c>
       <c r="D87" t="n">
-        <v>0.9954388417209628</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="88">
@@ -1665,7 +1665,7 @@
         <v>58.69657861547959</v>
       </c>
       <c r="D88" t="n">
-        <v>0.9944233499910683</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="89">
@@ -1679,7 +1679,7 @@
         <v>38.56371252741226</v>
       </c>
       <c r="D89" t="n">
-        <v>0.9954124390920636</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="90">
@@ -1693,7 +1693,7 @@
         <v>52.50241733428958</v>
       </c>
       <c r="D90" t="n">
-        <v>0.9950762147747898</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="91">
@@ -1707,7 +1707,7 @@
         <v>36.73129929489149</v>
       </c>
       <c r="D91" t="n">
-        <v>0.9980141319746971</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="92">
@@ -1721,7 +1721,7 @@
         <v>38.354514288082</v>
       </c>
       <c r="D92" t="n">
-        <v>0.9982655717208354</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="93">
@@ -1735,7 +1735,7 @@
         <v>35.67810581622993</v>
       </c>
       <c r="D93" t="n">
-        <v>0.9916943144499213</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="94">
@@ -1749,7 +1749,7 @@
         <v>53.07213893313723</v>
       </c>
       <c r="D94" t="n">
-        <v>0.9984790878252348</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="95">
@@ -1763,7 +1763,7 @@
         <v>48.86920189220226</v>
       </c>
       <c r="D95" t="n">
-        <v>0.9970895396369051</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="96">
@@ -1777,7 +1777,7 @@
         <v>62.85358877955228</v>
       </c>
       <c r="D96" t="n">
-        <v>0.9957512362700067</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="97">
@@ -1791,7 +1791,7 @@
         <v>51.47706433991497</v>
       </c>
       <c r="D97" t="n">
-        <v>0.9959364654074185</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="98">
@@ -1805,7 +1805,7 @@
         <v>62.72713000736199</v>
       </c>
       <c r="D98" t="n">
-        <v>0.9949145420691058</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="99">
@@ -1819,7 +1819,7 @@
         <v>30.1299770846383</v>
       </c>
       <c r="D99" t="n">
-        <v>0.9982553696967855</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="100">
@@ -1833,7 +1833,7 @@
         <v>36.75800440157938</v>
       </c>
       <c r="D100" t="n">
-        <v>0.9920993688558012</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="101">
@@ -1847,7 +1847,7 @@
         <v>63.89390408530792</v>
       </c>
       <c r="D101" t="n">
-        <v>0.9953938439304262</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="102">
@@ -1861,7 +1861,7 @@
         <v>26.79910170703495</v>
       </c>
       <c r="D102" t="n">
-        <v>0.9973281875568448</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="103">
@@ -1875,7 +1875,7 @@
         <v>60.78466344124584</v>
       </c>
       <c r="D103" t="n">
-        <v>0.9912128530645902</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="104">
@@ -1889,7 +1889,7 @@
         <v>50.48567520359704</v>
       </c>
       <c r="D104" t="n">
-        <v>0.9955395744692298</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="105">
@@ -1903,7 +1903,7 @@
         <v>41.35935978814719</v>
       </c>
       <c r="D105" t="n">
-        <v>0.9936255012797661</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="106">
@@ -1917,7 +1917,7 @@
         <v>42.82388935866014</v>
       </c>
       <c r="D106" t="n">
-        <v>0.9968943270731966</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="107">
@@ -1931,7 +1931,7 @@
         <v>68.23917794835043</v>
       </c>
       <c r="D107" t="n">
-        <v>0.9906094292455848</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="108">
@@ -1945,7 +1945,7 @@
         <v>59.83732978424243</v>
       </c>
       <c r="D108" t="n">
-        <v>0.9954613294293079</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="109">
@@ -1959,7 +1959,7 @@
         <v>74.63434472715409</v>
       </c>
       <c r="D109" t="n">
-        <v>0.9977137082098798</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="110">
@@ -1973,7 +1973,7 @@
         <v>43.8272972250524</v>
       </c>
       <c r="D110" t="n">
-        <v>0.9956551307612678</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="111">
@@ -1987,7 +1987,7 @@
         <v>38.43265364638556</v>
       </c>
       <c r="D111" t="n">
-        <v>0.9928920392590816</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="112">
@@ -2001,7 +2001,7 @@
         <v>43.35818692272822</v>
       </c>
       <c r="D112" t="n">
-        <v>0.995902164503297</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="113">
@@ -2015,7 +2015,7 @@
         <v>38.24494164978585</v>
       </c>
       <c r="D113" t="n">
-        <v>0.9930433755846241</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="114">
@@ -2029,7 +2029,7 @@
         <v>63.72798095751364</v>
       </c>
       <c r="D114" t="n">
-        <v>0.9960173350956908</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="115">
@@ -2043,7 +2043,7 @@
         <v>67.53649305633806</v>
       </c>
       <c r="D115" t="n">
-        <v>0.9911550996129784</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="116">
@@ -2057,7 +2057,7 @@
         <v>32.72351644182054</v>
       </c>
       <c r="D116" t="n">
-        <v>0.992519925697763</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="117">
@@ -2071,7 +2071,7 @@
         <v>61.59257328408566</v>
       </c>
       <c r="D117" t="n">
-        <v>0.9902944654037722</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="118">
@@ -2085,7 +2085,7 @@
         <v>25.38818198523678</v>
       </c>
       <c r="D118" t="n">
-        <v>0.9907551845006642</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="119">
@@ -2099,7 +2099,7 @@
         <v>45.79677033582375</v>
       </c>
       <c r="D119" t="n">
-        <v>0.9949929265783486</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="120">
@@ -2113,7 +2113,7 @@
         <v>37.48719016337304</v>
       </c>
       <c r="D120" t="n">
-        <v>0.9920852839925307</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="121">
@@ -2127,7 +2127,7 @@
         <v>32.63044854100505</v>
       </c>
       <c r="D121" t="n">
-        <v>0.9946447432887395</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="122">
@@ -2141,7 +2141,7 @@
         <v>68.28707584039341</v>
       </c>
       <c r="D122" t="n">
-        <v>0.9959361257976556</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="123">
@@ -2155,7 +2155,7 @@
         <v>33.24305624591818</v>
       </c>
       <c r="D123" t="n">
-        <v>0.9979306756141457</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="124">
@@ -2169,7 +2169,7 @@
         <v>44.03556352239427</v>
       </c>
       <c r="D124" t="n">
-        <v>0.9931955491312968</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="125">
@@ -2183,7 +2183,7 @@
         <v>42.74363943603997</v>
       </c>
       <c r="D125" t="n">
-        <v>0.9928681106979487</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="126">
@@ -2197,7 +2197,7 @@
         <v>58.85095317494391</v>
       </c>
       <c r="D126" t="n">
-        <v>0.9928230006740743</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="127">
@@ -2211,7 +2211,7 @@
         <v>16.17394847958799</v>
       </c>
       <c r="D127" t="n">
-        <v>0.9910606468007196</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="128">
@@ -2225,7 +2225,7 @@
         <v>33.87766682607845</v>
       </c>
       <c r="D128" t="n">
-        <v>0.9959686502819154</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="129">
@@ -2239,7 +2239,7 @@
         <v>47.00209216877489</v>
       </c>
       <c r="D129" t="n">
-        <v>0.9973768912329349</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="130">
@@ -2253,7 +2253,7 @@
         <v>21.82843164035993</v>
       </c>
       <c r="D130" t="n">
-        <v>0.9942570437477669</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="131">
@@ -2267,7 +2267,7 @@
         <v>60.99389115413728</v>
       </c>
       <c r="D131" t="n">
-        <v>0.9950246765725369</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="132">
@@ -2281,7 +2281,7 @@
         <v>56.44673584598896</v>
       </c>
       <c r="D132" t="n">
-        <v>0.9986263210232605</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="133">
@@ -2295,7 +2295,7 @@
         <v>69.7668412155984</v>
       </c>
       <c r="D133" t="n">
-        <v>0.9962902365448724</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="134">
@@ -2309,7 +2309,7 @@
         <v>61.90100495581607</v>
       </c>
       <c r="D134" t="n">
-        <v>0.9967053139798289</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="135">
@@ -2323,7 +2323,7 @@
         <v>67.47581972462075</v>
       </c>
       <c r="D135" t="n">
-        <v>0.9980054852157407</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="136">
@@ -2337,7 +2337,7 @@
         <v>56.0214981912111</v>
       </c>
       <c r="D136" t="n">
-        <v>0.9919421151847571</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="137">
@@ -2351,7 +2351,7 @@
         <v>50.95247214583335</v>
       </c>
       <c r="D137" t="n">
-        <v>0.9958514945248862</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="138">
@@ -2365,7 +2365,7 @@
         <v>53.57551639207747</v>
       </c>
       <c r="D138" t="n">
-        <v>0.9964565505479376</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="139">
@@ -2379,7 +2379,7 @@
         <v>50.14878729140165</v>
       </c>
       <c r="D139" t="n">
-        <v>0.9975800513675117</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="140">
@@ -2393,7 +2393,7 @@
         <v>39.11919311989337</v>
       </c>
       <c r="D140" t="n">
-        <v>0.9930940699140171</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="141">
@@ -2407,7 +2407,7 @@
         <v>57.67393992818478</v>
       </c>
       <c r="D141" t="n">
-        <v>0.9961991523514174</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="142">
@@ -2421,7 +2421,7 @@
         <v>59.98976470976152</v>
       </c>
       <c r="D142" t="n">
-        <v>0.9954396054522234</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="143">
@@ -2435,7 +2435,7 @@
         <v>61.29403023760543</v>
       </c>
       <c r="D143" t="n">
-        <v>0.993684249304404</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="144">
@@ -2449,7 +2449,7 @@
         <v>41.06339365608342</v>
       </c>
       <c r="D144" t="n">
-        <v>0.9909151718137394</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="145">
@@ -2463,7 +2463,7 @@
         <v>71.71488219151669</v>
       </c>
       <c r="D145" t="n">
-        <v>0.9931774359040483</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="146">
@@ -2477,7 +2477,7 @@
         <v>33.21788065693907</v>
       </c>
       <c r="D146" t="n">
-        <v>0.9986713627330843</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="147">
@@ -2491,7 +2491,7 @@
         <v>35.76532379625473</v>
       </c>
       <c r="D147" t="n">
-        <v>0.9919487115145151</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="148">
@@ -2505,7 +2505,7 @@
         <v>50.30715431918719</v>
       </c>
       <c r="D148" t="n">
-        <v>0.9910227419422936</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="149">
@@ -2519,7 +2519,7 @@
         <v>41.70098183161208</v>
       </c>
       <c r="D149" t="n">
-        <v>0.9933091148226331</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="150">
@@ -2533,7 +2533,7 @@
         <v>25.71370826456232</v>
       </c>
       <c r="D150" t="n">
-        <v>0.9909088271289538</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="151">
@@ -2547,7 +2547,7 @@
         <v>26.49052869939182</v>
       </c>
       <c r="D151" t="n">
-        <v>0.9924047903865264</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="152">
@@ -2561,7 +2561,7 @@
         <v>63.90692432390129</v>
       </c>
       <c r="D152" t="n">
-        <v>0.9982301050989263</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="153">
@@ -2575,7 +2575,7 @@
         <v>63.37928648737845</v>
       </c>
       <c r="D153" t="n">
-        <v>0.9928690387330102</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="154">
@@ -2589,7 +2589,7 @@
         <v>25.12029222292051</v>
       </c>
       <c r="D154" t="n">
-        <v>0.9952730056309215</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="155">
@@ -2603,7 +2603,7 @@
         <v>39.60329258760133</v>
       </c>
       <c r="D155" t="n">
-        <v>0.9921487030159946</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="156">
@@ -2617,7 +2617,7 @@
         <v>12.21263075110782</v>
       </c>
       <c r="D156" t="n">
-        <v>0.9960118193195865</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="157">
@@ -2631,7 +2631,7 @@
         <v>30.54834043508056</v>
       </c>
       <c r="D157" t="n">
-        <v>0.991148907488984</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="158">
@@ -2645,7 +2645,7 @@
         <v>50.03149339688316</v>
       </c>
       <c r="D158" t="n">
-        <v>0.9971082844494795</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="159">
@@ -2659,7 +2659,7 @@
         <v>47.94394853399143</v>
       </c>
       <c r="D159" t="n">
-        <v>0.9938065144029443</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="160">
@@ -2673,7 +2673,7 @@
         <v>69.92956674357832</v>
       </c>
       <c r="D160" t="n">
-        <v>0.9916529434838228</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="161">
@@ -2687,7 +2687,7 @@
         <v>31.9704602093228</v>
       </c>
       <c r="D161" t="n">
-        <v>0.9968242460908364</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="162">
@@ -2701,7 +2701,7 @@
         <v>38.96577069630239</v>
       </c>
       <c r="D162" t="n">
-        <v>0.9949885428512451</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="163">
@@ -2715,7 +2715,7 @@
         <v>39.39751136993004</v>
       </c>
       <c r="D163" t="n">
-        <v>0.9939433050929787</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="164">
@@ -2729,7 +2729,7 @@
         <v>70.84264618277928</v>
       </c>
       <c r="D164" t="n">
-        <v>0.992165634376324</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="165">
@@ -2743,7 +2743,7 @@
         <v>33.99966038162763</v>
       </c>
       <c r="D165" t="n">
-        <v>0.9970322930387524</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="166">
@@ -2757,7 +2757,7 @@
         <v>56.52139609313584</v>
       </c>
       <c r="D166" t="n">
-        <v>0.9932875655103311</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="167">
@@ -2771,7 +2771,7 @@
         <v>51.63354419283532</v>
       </c>
       <c r="D167" t="n">
-        <v>0.9903878162157114</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="168">
@@ -2785,7 +2785,7 @@
         <v>47.10708506835977</v>
       </c>
       <c r="D168" t="n">
-        <v>0.9986883234286021</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="169">
@@ -2799,7 +2799,7 @@
         <v>55.25408342657246</v>
       </c>
       <c r="D169" t="n">
-        <v>0.990274183273124</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="170">
@@ -2813,7 +2813,7 @@
         <v>60.65846113009473</v>
       </c>
       <c r="D170" t="n">
-        <v>0.9910842216986149</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="171">
@@ -2827,7 +2827,7 @@
         <v>89.11758782502773</v>
       </c>
       <c r="D171" t="n">
-        <v>0.9941923127789584</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="172">
@@ -2841,7 +2841,7 @@
         <v>34.15141111167516</v>
       </c>
       <c r="D172" t="n">
-        <v>0.9918706944741474</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="173">
@@ -2855,7 +2855,7 @@
         <v>81.70343159249632</v>
       </c>
       <c r="D173" t="n">
-        <v>0.9930162153382749</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="174">
@@ -2869,7 +2869,7 @@
         <v>66.67672188427332</v>
       </c>
       <c r="D174" t="n">
-        <v>0.9951080871774001</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="175">
@@ -2883,7 +2883,7 @@
         <v>55.87154050616485</v>
       </c>
       <c r="D175" t="n">
-        <v>0.9986205775703306</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="176">
@@ -2897,7 +2897,7 @@
         <v>38.00322570895611</v>
       </c>
       <c r="D176" t="n">
-        <v>0.9984268100183206</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="177">
@@ -2911,7 +2911,7 @@
         <v>29.69824828000953</v>
       </c>
       <c r="D177" t="n">
-        <v>0.9906650637826071</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="178">
@@ -2925,7 +2925,7 @@
         <v>51.10642431092796</v>
       </c>
       <c r="D178" t="n">
-        <v>0.9976798229063399</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="179">
@@ -2939,7 +2939,7 @@
         <v>58.24256654083357</v>
       </c>
       <c r="D179" t="n">
-        <v>0.9915104128961902</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="180">
@@ -2953,7 +2953,7 @@
         <v>57.90753875284465</v>
       </c>
       <c r="D180" t="n">
-        <v>0.9973028958525291</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="181">
@@ -2967,7 +2967,7 @@
         <v>37.82288482564915</v>
       </c>
       <c r="D181" t="n">
-        <v>0.9926671249606338</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="182">
@@ -2981,7 +2981,7 @@
         <v>59.72710216882905</v>
       </c>
       <c r="D182" t="n">
-        <v>0.9964605092155461</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="183">
@@ -2995,7 +2995,7 @@
         <v>30.0882005832016</v>
       </c>
       <c r="D183" t="n">
-        <v>0.9964691388452478</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="184">
@@ -3009,7 +3009,7 @@
         <v>50.0340207885088</v>
       </c>
       <c r="D184" t="n">
-        <v>0.9976549613378072</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="185">
@@ -3023,7 +3023,7 @@
         <v>22.99356530034146</v>
       </c>
       <c r="D185" t="n">
-        <v>0.9988166326396635</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="186">
@@ -3037,7 +3037,7 @@
         <v>70.53643160720347</v>
       </c>
       <c r="D186" t="n">
-        <v>0.992479327675767</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="187">
@@ -3051,7 +3051,7 @@
         <v>69.30669020013021</v>
       </c>
       <c r="D187" t="n">
-        <v>0.9956547761280695</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="188">
@@ -3065,7 +3065,7 @@
         <v>53.28708600267237</v>
       </c>
       <c r="D188" t="n">
-        <v>0.9966533471607333</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="189">
@@ -3079,7 +3079,7 @@
         <v>58.33525434379268</v>
       </c>
       <c r="D189" t="n">
-        <v>0.9907166640381805</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="190">
@@ -3093,7 +3093,7 @@
         <v>52.21783588359124</v>
       </c>
       <c r="D190" t="n">
-        <v>0.9959666520399196</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="191">
@@ -3107,7 +3107,7 @@
         <v>73.04385275833977</v>
       </c>
       <c r="D191" t="n">
-        <v>0.9928936396377742</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="192">
@@ -3121,7 +3121,7 @@
         <v>47.88198415669979</v>
       </c>
       <c r="D192" t="n">
-        <v>0.9914532213839485</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="193">
@@ -3135,7 +3135,7 @@
         <v>31.82557362505747</v>
       </c>
       <c r="D193" t="n">
-        <v>0.9949452440205129</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="194">
@@ -3149,7 +3149,7 @@
         <v>7.703496491937528</v>
       </c>
       <c r="D194" t="n">
-        <v>0.9941569523736981</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="195">
@@ -3163,7 +3163,7 @@
         <v>57.38510043723399</v>
       </c>
       <c r="D195" t="n">
-        <v>0.9951937184966392</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="196">
@@ -3177,7 +3177,7 @@
         <v>21.07210778365031</v>
       </c>
       <c r="D196" t="n">
-        <v>0.9957772583136302</v>
+        <v>0.99</v>
       </c>
     </row>
     <row r="197">
@@ -3191,7 +3191,7 @@
         <v>50.77438967751996</v>
       </c>
       <c r="D197" t="n">
-        <v>0.9944880197521365</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="198">
@@ -3205,7 +3205,7 @@
         <v>59.94433851813749</v>
       </c>
       <c r="D198" t="n">
-        <v>0.9981463563669523</v>
+        <v>0.999</v>
       </c>
     </row>
     <row r="199">
@@ -3219,7 +3219,7 @@
         <v>18.08351560802339</v>
       </c>
       <c r="D199" t="n">
-        <v>0.9916012277855191</v>
+        <v>0.9999</v>
       </c>
     </row>
     <row r="200">
@@ -3233,7 +3233,7 @@
         <v>48.88290551241017</v>
       </c>
       <c r="D200" t="n">
-        <v>0.9925991248410848</v>
+        <v>0.9</v>
       </c>
     </row>
     <row r="201">
@@ -3247,7 +3247,7 @@
         <v>60.19400006076078</v>
       </c>
       <c r="D201" t="n">
-        <v>0.9932059947706208</v>
+        <v>0.9999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add reliability-constrained QoS scheduling and four-method experiments
Integrate GH reliability, masked PPO with completion-interval effective QoS, task deadlines, TORE/RASOUL baselines, unified metrics, and reproducible paired experiments. Include task inputs, documentation, and tests; exclude generated experiment outputs and model checkpoints.
</commit_message>
<xml_diff>
--- a/data/task_parameters.xlsx
+++ b/data/task_parameters.xlsx
@@ -16,7 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +57,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D201"/>
+  <dimension ref="A1:E201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,6 +452,11 @@
           <t>Reliability_Requirement</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Deadline</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -463,6 +471,9 @@
       <c r="D2" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E2" s="2" t="n">
+        <v>1.719694235101399</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -475,7 +486,10 @@
         <v>3615434722.997388</v>
       </c>
       <c r="D3" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>2.103070748639826</v>
       </c>
     </row>
     <row r="4">
@@ -491,6 +505,9 @@
       <c r="D4" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E4" s="2" t="n">
+        <v>2.066076611076461</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -503,7 +520,10 @@
         <v>3221652678.905345</v>
       </c>
       <c r="D5" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>1.864840898232489</v>
       </c>
     </row>
     <row r="6">
@@ -519,6 +539,9 @@
       <c r="D6" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E6" s="2" t="n">
+        <v>1.857273883847675</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -531,7 +554,10 @@
         <v>3786745981.1374</v>
       </c>
       <c r="D7" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>2.147910769241209</v>
       </c>
     </row>
     <row r="8">
@@ -545,7 +571,10 @@
         <v>2499438637.785756</v>
       </c>
       <c r="D8" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>1.634314941012166</v>
       </c>
     </row>
     <row r="9">
@@ -559,7 +588,10 @@
         <v>2943268450.966835</v>
       </c>
       <c r="D9" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>1.718257775931188</v>
       </c>
     </row>
     <row r="10">
@@ -575,6 +607,9 @@
       <c r="D10" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E10" s="2" t="n">
+        <v>1.512285654411353</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -587,7 +622,10 @@
         <v>3614211371.093409</v>
       </c>
       <c r="D11" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>1.823646807345262</v>
       </c>
     </row>
     <row r="12">
@@ -603,6 +641,9 @@
       <c r="D12" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E12" s="2" t="n">
+        <v>1.738202911077727</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -615,7 +656,10 @@
         <v>2512625659.984993</v>
       </c>
       <c r="D13" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>1.675001363896212</v>
       </c>
     </row>
     <row r="14">
@@ -629,7 +673,10 @@
         <v>2113145785.68241</v>
       </c>
       <c r="D14" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>1.22967806569779</v>
       </c>
     </row>
     <row r="15">
@@ -645,6 +692,9 @@
       <c r="D15" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E15" s="2" t="n">
+        <v>1.332178001947635</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -657,7 +707,10 @@
         <v>3253200261.046153</v>
       </c>
       <c r="D16" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>1.989511073654613</v>
       </c>
     </row>
     <row r="17">
@@ -671,7 +724,10 @@
         <v>2035734367.391731</v>
       </c>
       <c r="D17" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>1.274682267944549</v>
       </c>
     </row>
     <row r="18">
@@ -687,6 +743,9 @@
       <c r="D18" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E18" s="2" t="n">
+        <v>1.862003118176583</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -699,7 +758,10 @@
         <v>3944878070.402884</v>
       </c>
       <c r="D19" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>1.970881325016217</v>
       </c>
     </row>
     <row r="20">
@@ -713,7 +775,10 @@
         <v>2756814765.212242</v>
       </c>
       <c r="D20" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>1.590541130959746</v>
       </c>
     </row>
     <row r="21">
@@ -729,6 +794,9 @@
       <c r="D21" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E21" s="2" t="n">
+        <v>2.140301332293814</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -743,6 +811,9 @@
       <c r="D22" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E22" s="2" t="n">
+        <v>1.695460727095932</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -755,7 +826,10 @@
         <v>2379578199.105142</v>
       </c>
       <c r="D23" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>1.370998844757819</v>
       </c>
     </row>
     <row r="24">
@@ -769,7 +843,10 @@
         <v>2475034639.987186</v>
       </c>
       <c r="D24" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>1.571033915180994</v>
       </c>
     </row>
     <row r="25">
@@ -783,7 +860,10 @@
         <v>3320683924.82158</v>
       </c>
       <c r="D25" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>1.655003308239766</v>
       </c>
     </row>
     <row r="26">
@@ -797,7 +877,10 @@
         <v>3789278080.928905</v>
       </c>
       <c r="D26" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E26" s="2" t="n">
+        <v>2.154511438074283</v>
       </c>
     </row>
     <row r="27">
@@ -811,7 +894,10 @@
         <v>2809540495.200351</v>
       </c>
       <c r="D27" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>1.566016176970736</v>
       </c>
     </row>
     <row r="28">
@@ -827,6 +913,9 @@
       <c r="D28" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E28" s="2" t="n">
+        <v>1.587996509894193</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -839,7 +928,10 @@
         <v>3883961950.771987</v>
       </c>
       <c r="D29" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>2.111341816933927</v>
       </c>
     </row>
     <row r="30">
@@ -855,6 +947,9 @@
       <c r="D30" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E30" s="2" t="n">
+        <v>1.511388355924895</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -867,7 +962,10 @@
         <v>3849467486.215332</v>
       </c>
       <c r="D31" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>2.160840366858225</v>
       </c>
     </row>
     <row r="32">
@@ -881,7 +979,10 @@
         <v>2572845237.661914</v>
       </c>
       <c r="D32" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E32" s="2" t="n">
+        <v>1.439480782917656</v>
       </c>
     </row>
     <row r="33">
@@ -897,6 +998,9 @@
       <c r="D33" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E33" s="2" t="n">
+        <v>1.899990441963975</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -909,7 +1013,10 @@
         <v>2137930559.569284</v>
       </c>
       <c r="D34" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E34" s="2" t="n">
+        <v>1.411385117263159</v>
       </c>
     </row>
     <row r="35">
@@ -923,7 +1030,10 @@
         <v>3343164810.637867</v>
       </c>
       <c r="D35" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>1.865577410347485</v>
       </c>
     </row>
     <row r="36">
@@ -939,6 +1049,9 @@
       <c r="D36" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E36" s="2" t="n">
+        <v>1.524224658512922</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -951,7 +1064,10 @@
         <v>2943833942.691082</v>
       </c>
       <c r="D37" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>1.757027068393899</v>
       </c>
     </row>
     <row r="38">
@@ -965,7 +1081,10 @@
         <v>2710788763.434069</v>
       </c>
       <c r="D38" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E38" s="2" t="n">
+        <v>1.748954426697872</v>
       </c>
     </row>
     <row r="39">
@@ -979,7 +1098,10 @@
         <v>2274241911.740644</v>
       </c>
       <c r="D39" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>1.311702126598665</v>
       </c>
     </row>
     <row r="40">
@@ -993,7 +1115,10 @@
         <v>2830705215.863926</v>
       </c>
       <c r="D40" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E40" s="2" t="n">
+        <v>1.82775480308597</v>
       </c>
     </row>
     <row r="41">
@@ -1007,7 +1132,10 @@
         <v>2805627574.532079</v>
       </c>
       <c r="D41" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>1.710747679972703</v>
       </c>
     </row>
     <row r="42">
@@ -1021,7 +1149,10 @@
         <v>2909373830.98064</v>
       </c>
       <c r="D42" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E42" s="2" t="n">
+        <v>1.547752310732462</v>
       </c>
     </row>
     <row r="43">
@@ -1035,7 +1166,10 @@
         <v>3727776757.362188</v>
       </c>
       <c r="D43" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>2.175018830908277</v>
       </c>
     </row>
     <row r="44">
@@ -1049,7 +1183,10 @@
         <v>2595320155.771381</v>
       </c>
       <c r="D44" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E44" s="2" t="n">
+        <v>1.500634439867138</v>
       </c>
     </row>
     <row r="45">
@@ -1063,7 +1200,10 @@
         <v>2229907194.491547</v>
       </c>
       <c r="D45" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>1.360350519348226</v>
       </c>
     </row>
     <row r="46">
@@ -1077,7 +1217,10 @@
         <v>2781107413.213808</v>
       </c>
       <c r="D46" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E46" s="2" t="n">
+        <v>1.820825965984033</v>
       </c>
     </row>
     <row r="47">
@@ -1091,7 +1234,10 @@
         <v>3871586029.915329</v>
       </c>
       <c r="D47" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E47" s="2" t="n">
+        <v>1.961774718575748</v>
       </c>
     </row>
     <row r="48">
@@ -1105,7 +1251,10 @@
         <v>2844478785.842661</v>
       </c>
       <c r="D48" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E48" s="2" t="n">
+        <v>1.513637642760613</v>
       </c>
     </row>
     <row r="49">
@@ -1119,7 +1268,10 @@
         <v>2507596881.018478</v>
       </c>
       <c r="D49" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E49" s="2" t="n">
+        <v>1.44681992967971</v>
       </c>
     </row>
     <row r="50">
@@ -1133,7 +1285,10 @@
         <v>3124406713.111102</v>
       </c>
       <c r="D50" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E50" s="2" t="n">
+        <v>1.593960088764917</v>
       </c>
     </row>
     <row r="51">
@@ -1147,7 +1302,10 @@
         <v>3594487309.937557</v>
       </c>
       <c r="D51" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E51" s="2" t="n">
+        <v>1.854498841039235</v>
       </c>
     </row>
     <row r="52">
@@ -1161,7 +1319,10 @@
         <v>3510304661.60333</v>
       </c>
       <c r="D52" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E52" s="2" t="n">
+        <v>2.1018171045938</v>
       </c>
     </row>
     <row r="53">
@@ -1175,7 +1336,10 @@
         <v>3554514302.615196</v>
       </c>
       <c r="D53" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E53" s="2" t="n">
+        <v>1.883580292177504</v>
       </c>
     </row>
     <row r="54">
@@ -1189,7 +1353,10 @@
         <v>3875271685.39693</v>
       </c>
       <c r="D54" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E54" s="2" t="n">
+        <v>2.03889743542455</v>
       </c>
     </row>
     <row r="55">
@@ -1203,7 +1370,10 @@
         <v>3802214158.329295</v>
       </c>
       <c r="D55" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E55" s="2" t="n">
+        <v>1.831632936029274</v>
       </c>
     </row>
     <row r="56">
@@ -1217,7 +1387,10 @@
         <v>2541560741.546412</v>
       </c>
       <c r="D56" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E56" s="2" t="n">
+        <v>1.570875995675674</v>
       </c>
     </row>
     <row r="57">
@@ -1231,7 +1404,10 @@
         <v>3604878363.624515</v>
       </c>
       <c r="D57" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E57" s="2" t="n">
+        <v>2.000996063099563</v>
       </c>
     </row>
     <row r="58">
@@ -1245,7 +1421,10 @@
         <v>2436981573.833116</v>
       </c>
       <c r="D58" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E58" s="2" t="n">
+        <v>1.439631861791494</v>
       </c>
     </row>
     <row r="59">
@@ -1259,7 +1438,10 @@
         <v>2980335627.828416</v>
       </c>
       <c r="D59" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E59" s="2" t="n">
+        <v>1.782733673506268</v>
       </c>
     </row>
     <row r="60">
@@ -1273,7 +1455,10 @@
         <v>2851571343.884669</v>
       </c>
       <c r="D60" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E60" s="2" t="n">
+        <v>1.739310100917165</v>
       </c>
     </row>
     <row r="61">
@@ -1287,7 +1472,10 @@
         <v>3431132069.789394</v>
       </c>
       <c r="D61" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E61" s="2" t="n">
+        <v>1.904414560838833</v>
       </c>
     </row>
     <row r="62">
@@ -1301,7 +1489,10 @@
         <v>2153053396.488575</v>
       </c>
       <c r="D62" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E62" s="2" t="n">
+        <v>1.38532373962597</v>
       </c>
     </row>
     <row r="63">
@@ -1317,6 +1508,9 @@
       <c r="D63" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E63" s="2" t="n">
+        <v>1.53338990482089</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1329,7 +1523,10 @@
         <v>3130182437.904866</v>
       </c>
       <c r="D64" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E64" s="2" t="n">
+        <v>1.877421206055043</v>
       </c>
     </row>
     <row r="65">
@@ -1345,6 +1542,9 @@
       <c r="D65" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E65" s="2" t="n">
+        <v>2.231579613852943</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1359,6 +1559,9 @@
       <c r="D66" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E66" s="2" t="n">
+        <v>1.948383908574805</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1373,6 +1576,9 @@
       <c r="D67" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E67" s="2" t="n">
+        <v>1.523676813073203</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1385,7 +1591,10 @@
         <v>3335371620.389873</v>
       </c>
       <c r="D68" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E68" s="2" t="n">
+        <v>1.915280984070574</v>
       </c>
     </row>
     <row r="69">
@@ -1401,6 +1610,9 @@
       <c r="D69" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E69" s="2" t="n">
+        <v>1.513845785614459</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1413,7 +1625,10 @@
         <v>3824515162.420707</v>
       </c>
       <c r="D70" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E70" s="2" t="n">
+        <v>2.130850914236655</v>
       </c>
     </row>
     <row r="71">
@@ -1427,7 +1642,10 @@
         <v>2909476483.135699</v>
       </c>
       <c r="D71" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E71" s="2" t="n">
+        <v>1.791182342261058</v>
       </c>
     </row>
     <row r="72">
@@ -1441,7 +1659,10 @@
         <v>2241819552.432022</v>
       </c>
       <c r="D72" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E72" s="2" t="n">
+        <v>1.274980209511935</v>
       </c>
     </row>
     <row r="73">
@@ -1457,6 +1678,9 @@
       <c r="D73" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E73" s="2" t="n">
+        <v>1.639935614684337</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -1469,7 +1693,10 @@
         <v>3386717624.178626</v>
       </c>
       <c r="D74" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E74" s="2" t="n">
+        <v>1.919642695117606</v>
       </c>
     </row>
     <row r="75">
@@ -1485,6 +1712,9 @@
       <c r="D75" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E75" s="2" t="n">
+        <v>1.292099298423033</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -1497,7 +1727,10 @@
         <v>3165213918.953576</v>
       </c>
       <c r="D76" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E76" s="2" t="n">
+        <v>1.77693114965838</v>
       </c>
     </row>
     <row r="77">
@@ -1511,7 +1744,10 @@
         <v>3503060116.091953</v>
       </c>
       <c r="D77" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E77" s="2" t="n">
+        <v>1.791706911855619</v>
       </c>
     </row>
     <row r="78">
@@ -1525,7 +1761,10 @@
         <v>3091240503.911071</v>
       </c>
       <c r="D78" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E78" s="2" t="n">
+        <v>1.657460481077803</v>
       </c>
     </row>
     <row r="79">
@@ -1541,6 +1780,9 @@
       <c r="D79" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E79" s="2" t="n">
+        <v>1.364337762302086</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -1555,6 +1797,9 @@
       <c r="D80" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E80" s="2" t="n">
+        <v>2.018546018086391</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -1567,7 +1812,10 @@
         <v>3803942783.409199</v>
       </c>
       <c r="D81" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E81" s="2" t="n">
+        <v>1.83710522565812</v>
       </c>
     </row>
     <row r="82">
@@ -1581,7 +1829,10 @@
         <v>2103803148.624906</v>
       </c>
       <c r="D82" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E82" s="2" t="n">
+        <v>1.335086962852651</v>
       </c>
     </row>
     <row r="83">
@@ -1595,7 +1846,10 @@
         <v>3265033710.779034</v>
       </c>
       <c r="D83" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E83" s="2" t="n">
+        <v>1.623895630345506</v>
       </c>
     </row>
     <row r="84">
@@ -1609,7 +1863,10 @@
         <v>2287977748.73364</v>
       </c>
       <c r="D84" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E84" s="2" t="n">
+        <v>1.442657960948069</v>
       </c>
     </row>
     <row r="85">
@@ -1625,6 +1882,9 @@
       <c r="D85" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E85" s="2" t="n">
+        <v>1.88649520991912</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -1637,7 +1897,10 @@
         <v>2183793613.868398</v>
       </c>
       <c r="D86" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E86" s="2" t="n">
+        <v>1.333571961680017</v>
       </c>
     </row>
     <row r="87">
@@ -1651,7 +1914,10 @@
         <v>3943469311.840803</v>
       </c>
       <c r="D87" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E87" s="2" t="n">
+        <v>1.942625488401806</v>
       </c>
     </row>
     <row r="88">
@@ -1665,7 +1931,10 @@
         <v>3368310877.429912</v>
       </c>
       <c r="D88" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E88" s="2" t="n">
+        <v>1.830488786913041</v>
       </c>
     </row>
     <row r="89">
@@ -1679,7 +1948,10 @@
         <v>3895399651.296702</v>
       </c>
       <c r="D89" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E89" s="2" t="n">
+        <v>2.192184183393362</v>
       </c>
     </row>
     <row r="90">
@@ -1693,7 +1965,10 @@
         <v>3039261647.747734</v>
       </c>
       <c r="D90" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E90" s="2" t="n">
+        <v>1.56714263314985</v>
       </c>
     </row>
     <row r="91">
@@ -1707,7 +1982,10 @@
         <v>3057513183.274941</v>
       </c>
       <c r="D91" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E91" s="2" t="n">
+        <v>1.667468353797976</v>
       </c>
     </row>
     <row r="92">
@@ -1721,7 +1999,10 @@
         <v>3711030187.769846</v>
       </c>
       <c r="D92" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E92" s="2" t="n">
+        <v>1.957470338155397</v>
       </c>
     </row>
     <row r="93">
@@ -1735,7 +2016,10 @@
         <v>2721945784.562086</v>
       </c>
       <c r="D93" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E93" s="2" t="n">
+        <v>1.564348318529679</v>
       </c>
     </row>
     <row r="94">
@@ -1751,6 +2035,9 @@
       <c r="D94" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E94" s="2" t="n">
+        <v>1.876106702013563</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -1763,7 +2050,10 @@
         <v>2619582340.477922</v>
       </c>
       <c r="D95" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E95" s="2" t="n">
+        <v>1.749252810105866</v>
       </c>
     </row>
     <row r="96">
@@ -1777,7 +2067,10 @@
         <v>3264635626.331596</v>
       </c>
       <c r="D96" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E96" s="2" t="n">
+        <v>1.824693371543763</v>
       </c>
     </row>
     <row r="97">
@@ -1791,7 +2084,10 @@
         <v>2597651623.571331</v>
       </c>
       <c r="D97" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E97" s="2" t="n">
+        <v>1.516906684516891</v>
       </c>
     </row>
     <row r="98">
@@ -1807,6 +2103,9 @@
       <c r="D98" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E98" s="2" t="n">
+        <v>1.60885460484537</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -1819,7 +2118,10 @@
         <v>3313890175.43737</v>
       </c>
       <c r="D99" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E99" s="2" t="n">
+        <v>1.746134444904799</v>
       </c>
     </row>
     <row r="100">
@@ -1833,7 +2135,10 @@
         <v>2917070134.366358</v>
       </c>
       <c r="D100" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E100" s="2" t="n">
+        <v>1.783768655377179</v>
       </c>
     </row>
     <row r="101">
@@ -1847,7 +2152,10 @@
         <v>3295654151.10424</v>
       </c>
       <c r="D101" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E101" s="2" t="n">
+        <v>2.003025111112419</v>
       </c>
     </row>
     <row r="102">
@@ -1861,7 +2169,10 @@
         <v>3020248282.319529</v>
       </c>
       <c r="D102" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E102" s="2" t="n">
+        <v>1.855923438117526</v>
       </c>
     </row>
     <row r="103">
@@ -1877,6 +2188,9 @@
       <c r="D103" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E103" s="2" t="n">
+        <v>1.469233851680327</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -1889,7 +2203,10 @@
         <v>3234449309.212807</v>
       </c>
       <c r="D104" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E104" s="2" t="n">
+        <v>1.86965345030952</v>
       </c>
     </row>
     <row r="105">
@@ -1903,7 +2220,10 @@
         <v>2049915326.81772</v>
       </c>
       <c r="D105" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E105" s="2" t="n">
+        <v>1.497952796883882</v>
       </c>
     </row>
     <row r="106">
@@ -1919,6 +2239,9 @@
       <c r="D106" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E106" s="2" t="n">
+        <v>1.617057688532235</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -1931,7 +2254,10 @@
         <v>2321195921.23542</v>
       </c>
       <c r="D107" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E107" s="2" t="n">
+        <v>1.312190334234292</v>
       </c>
     </row>
     <row r="108">
@@ -1947,6 +2273,9 @@
       <c r="D108" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E108" s="2" t="n">
+        <v>1.454000307939721</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -1959,7 +2288,10 @@
         <v>3071587269.52985</v>
       </c>
       <c r="D109" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E109" s="2" t="n">
+        <v>1.724779271446546</v>
       </c>
     </row>
     <row r="110">
@@ -1973,7 +2305,10 @@
         <v>3457575187.214504</v>
       </c>
       <c r="D110" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E110" s="2" t="n">
+        <v>2.010614224627431</v>
       </c>
     </row>
     <row r="111">
@@ -1989,6 +2324,9 @@
       <c r="D111" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E111" s="2" t="n">
+        <v>2.025828397368303</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2003,6 +2341,9 @@
       <c r="D112" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E112" s="2" t="n">
+        <v>1.439951006932654</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -2017,6 +2358,9 @@
       <c r="D113" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E113" s="2" t="n">
+        <v>1.629711622821386</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -2031,6 +2375,9 @@
       <c r="D114" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E114" s="2" t="n">
+        <v>1.6430258341687</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -2043,7 +2390,10 @@
         <v>2623330911.055835</v>
       </c>
       <c r="D115" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E115" s="2" t="n">
+        <v>1.624680176092834</v>
       </c>
     </row>
     <row r="116">
@@ -2059,6 +2409,9 @@
       <c r="D116" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E116" s="2" t="n">
+        <v>1.39864687530184</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -2071,7 +2424,10 @@
         <v>3809330131.554121</v>
       </c>
       <c r="D117" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E117" s="2" t="n">
+        <v>1.991184513787618</v>
       </c>
     </row>
     <row r="118">
@@ -2085,7 +2441,10 @@
         <v>3525043034.392427</v>
       </c>
       <c r="D118" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E118" s="2" t="n">
+        <v>2.063194095597995</v>
       </c>
     </row>
     <row r="119">
@@ -2099,7 +2458,10 @@
         <v>2087635256.409148</v>
       </c>
       <c r="D119" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E119" s="2" t="n">
+        <v>1.289451848794991</v>
       </c>
     </row>
     <row r="120">
@@ -2113,7 +2475,10 @@
         <v>3302044412.483964</v>
       </c>
       <c r="D120" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E120" s="2" t="n">
+        <v>1.827688663778707</v>
       </c>
     </row>
     <row r="121">
@@ -2127,7 +2492,10 @@
         <v>2279830186.2379</v>
       </c>
       <c r="D121" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E121" s="2" t="n">
+        <v>1.439046088216645</v>
       </c>
     </row>
     <row r="122">
@@ -2141,7 +2509,10 @@
         <v>2521993070.654481</v>
       </c>
       <c r="D122" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E122" s="2" t="n">
+        <v>1.675159699768785</v>
       </c>
     </row>
     <row r="123">
@@ -2155,7 +2526,10 @@
         <v>3185270236.053452</v>
       </c>
       <c r="D123" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E123" s="2" t="n">
+        <v>1.650206936003957</v>
       </c>
     </row>
     <row r="124">
@@ -2169,7 +2543,10 @@
         <v>2605453681.324949</v>
       </c>
       <c r="D124" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E124" s="2" t="n">
+        <v>1.377634082975438</v>
       </c>
     </row>
     <row r="125">
@@ -2183,7 +2560,10 @@
         <v>2229294466.610596</v>
       </c>
       <c r="D125" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E125" s="2" t="n">
+        <v>1.587678028574369</v>
       </c>
     </row>
     <row r="126">
@@ -2197,7 +2577,10 @@
         <v>3235001798.642087</v>
       </c>
       <c r="D126" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E126" s="2" t="n">
+        <v>1.657931568487654</v>
       </c>
     </row>
     <row r="127">
@@ -2213,6 +2596,9 @@
       <c r="D127" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E127" s="2" t="n">
+        <v>1.783655981979978</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -2225,7 +2611,10 @@
         <v>2588293930.618646</v>
       </c>
       <c r="D128" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E128" s="2" t="n">
+        <v>1.405229512519217</v>
       </c>
     </row>
     <row r="129">
@@ -2239,7 +2628,10 @@
         <v>2524084930.846177</v>
       </c>
       <c r="D129" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E129" s="2" t="n">
+        <v>1.7062985490375</v>
       </c>
     </row>
     <row r="130">
@@ -2253,7 +2645,10 @@
         <v>2998736000.999851</v>
       </c>
       <c r="D130" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E130" s="2" t="n">
+        <v>1.551790344590768</v>
       </c>
     </row>
     <row r="131">
@@ -2267,7 +2662,10 @@
         <v>3022939108.503745</v>
       </c>
       <c r="D131" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E131" s="2" t="n">
+        <v>1.795426910533304</v>
       </c>
     </row>
     <row r="132">
@@ -2281,7 +2679,10 @@
         <v>3685150274.072979</v>
       </c>
       <c r="D132" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E132" s="2" t="n">
+        <v>1.961183862436965</v>
       </c>
     </row>
     <row r="133">
@@ -2297,6 +2698,9 @@
       <c r="D133" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E133" s="2" t="n">
+        <v>1.774747755833276</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -2309,7 +2713,10 @@
         <v>3200612586.36801</v>
       </c>
       <c r="D134" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E134" s="2" t="n">
+        <v>1.96637149708936</v>
       </c>
     </row>
     <row r="135">
@@ -2323,7 +2730,10 @@
         <v>3990741212.238034</v>
       </c>
       <c r="D135" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E135" s="2" t="n">
+        <v>2.270670219863999</v>
       </c>
     </row>
     <row r="136">
@@ -2339,6 +2749,9 @@
       <c r="D136" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E136" s="2" t="n">
+        <v>1.623233800318796</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -2353,6 +2766,9 @@
       <c r="D137" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E137" s="2" t="n">
+        <v>1.873120851367485</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -2367,6 +2783,9 @@
       <c r="D138" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E138" s="2" t="n">
+        <v>2.087968645947611</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -2379,7 +2798,10 @@
         <v>2634964606.529172</v>
       </c>
       <c r="D139" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E139" s="2" t="n">
+        <v>1.643521406777116</v>
       </c>
     </row>
     <row r="140">
@@ -2393,7 +2815,10 @@
         <v>2325390109.876773</v>
       </c>
       <c r="D140" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E140" s="2" t="n">
+        <v>1.482972520848495</v>
       </c>
     </row>
     <row r="141">
@@ -2407,7 +2832,10 @@
         <v>3511092775.368326</v>
       </c>
       <c r="D141" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E141" s="2" t="n">
+        <v>1.768496808637778</v>
       </c>
     </row>
     <row r="142">
@@ -2421,7 +2849,10 @@
         <v>3516708830.245605</v>
       </c>
       <c r="D142" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E142" s="2" t="n">
+        <v>2.067815951956752</v>
       </c>
     </row>
     <row r="143">
@@ -2435,7 +2866,10 @@
         <v>2211024555.724195</v>
       </c>
       <c r="D143" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E143" s="2" t="n">
+        <v>1.574758704067134</v>
       </c>
     </row>
     <row r="144">
@@ -2449,7 +2883,10 @@
         <v>3961749000.019118</v>
       </c>
       <c r="D144" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E144" s="2" t="n">
+        <v>2.214226279935756</v>
       </c>
     </row>
     <row r="145">
@@ -2463,7 +2900,10 @@
         <v>3787693474.256113</v>
       </c>
       <c r="D145" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E145" s="2" t="n">
+        <v>2.160231986281822</v>
       </c>
     </row>
     <row r="146">
@@ -2477,7 +2917,10 @@
         <v>2318849594.271571</v>
       </c>
       <c r="D146" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E146" s="2" t="n">
+        <v>1.456089764867709</v>
       </c>
     </row>
     <row r="147">
@@ -2493,6 +2936,9 @@
       <c r="D147" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E147" s="2" t="n">
+        <v>1.800742694591331</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -2507,6 +2953,9 @@
       <c r="D148" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E148" s="2" t="n">
+        <v>1.505928827258459</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -2519,7 +2968,10 @@
         <v>2935624434.231703</v>
       </c>
       <c r="D149" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E149" s="2" t="n">
+        <v>1.511128717635713</v>
       </c>
     </row>
     <row r="150">
@@ -2533,7 +2985,10 @@
         <v>2272590775.494435</v>
       </c>
       <c r="D150" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E150" s="2" t="n">
+        <v>1.300881160873738</v>
       </c>
     </row>
     <row r="151">
@@ -2547,7 +3002,10 @@
         <v>2193525407.522423</v>
       </c>
       <c r="D151" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E151" s="2" t="n">
+        <v>1.509051316202543</v>
       </c>
     </row>
     <row r="152">
@@ -2561,7 +3019,10 @@
         <v>3489490288.600853</v>
       </c>
       <c r="D152" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E152" s="2" t="n">
+        <v>1.727688945247604</v>
       </c>
     </row>
     <row r="153">
@@ -2575,7 +3036,10 @@
         <v>3726087597.998542</v>
       </c>
       <c r="D153" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E153" s="2" t="n">
+        <v>2.179189594183646</v>
       </c>
     </row>
     <row r="154">
@@ -2589,7 +3053,10 @@
         <v>2112362513.782524</v>
       </c>
       <c r="D154" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E154" s="2" t="n">
+        <v>1.346370498601809</v>
       </c>
     </row>
     <row r="155">
@@ -2603,7 +3070,10 @@
         <v>3907450414.778891</v>
       </c>
       <c r="D155" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E155" s="2" t="n">
+        <v>2.222941248427873</v>
       </c>
     </row>
     <row r="156">
@@ -2619,6 +3089,9 @@
       <c r="D156" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E156" s="2" t="n">
+        <v>2.062405258903069</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -2633,6 +3106,9 @@
       <c r="D157" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E157" s="2" t="n">
+        <v>1.524976891795327</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -2645,7 +3121,10 @@
         <v>3909363009.374259</v>
       </c>
       <c r="D158" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E158" s="2" t="n">
+        <v>2.071090872713654</v>
       </c>
     </row>
     <row r="159">
@@ -2659,7 +3138,10 @@
         <v>2748041799.16139</v>
       </c>
       <c r="D159" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E159" s="2" t="n">
+        <v>1.443860959912037</v>
       </c>
     </row>
     <row r="160">
@@ -2673,7 +3155,10 @@
         <v>3175239088.345665</v>
       </c>
       <c r="D160" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E160" s="2" t="n">
+        <v>1.746865948649007</v>
       </c>
     </row>
     <row r="161">
@@ -2687,7 +3172,10 @@
         <v>3527518347.875824</v>
       </c>
       <c r="D161" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E161" s="2" t="n">
+        <v>2.008790657092171</v>
       </c>
     </row>
     <row r="162">
@@ -2701,7 +3189,10 @@
         <v>2867211109.095093</v>
       </c>
       <c r="D162" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E162" s="2" t="n">
+        <v>1.482074615936299</v>
       </c>
     </row>
     <row r="163">
@@ -2717,6 +3208,9 @@
       <c r="D163" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E163" s="2" t="n">
+        <v>1.844684324495937</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -2729,7 +3223,10 @@
         <v>2257174626.206392</v>
       </c>
       <c r="D164" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E164" s="2" t="n">
+        <v>1.509109324532123</v>
       </c>
     </row>
     <row r="165">
@@ -2743,7 +3240,10 @@
         <v>3507510245.45727</v>
       </c>
       <c r="D165" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E165" s="2" t="n">
+        <v>2.015489252767078</v>
       </c>
     </row>
     <row r="166">
@@ -2759,6 +3259,9 @@
       <c r="D166" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E166" s="2" t="n">
+        <v>1.492559434431366</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -2773,6 +3276,9 @@
       <c r="D167" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E167" s="2" t="n">
+        <v>1.736132023481587</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -2785,7 +3291,10 @@
         <v>3387143829.009998</v>
       </c>
       <c r="D168" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E168" s="2" t="n">
+        <v>1.738664122502986</v>
       </c>
     </row>
     <row r="169">
@@ -2801,6 +3310,9 @@
       <c r="D169" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E169" s="2" t="n">
+        <v>1.24626112400892</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -2813,7 +3325,10 @@
         <v>2247491917.743874</v>
       </c>
       <c r="D170" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E170" s="2" t="n">
+        <v>1.534029765828179</v>
       </c>
     </row>
     <row r="171">
@@ -2829,6 +3344,9 @@
       <c r="D171" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E171" s="2" t="n">
+        <v>1.541567898792439</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -2841,7 +3359,10 @@
         <v>2087114454.886926</v>
       </c>
       <c r="D172" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E172" s="2" t="n">
+        <v>1.571457343368644</v>
       </c>
     </row>
     <row r="173">
@@ -2855,7 +3376,10 @@
         <v>2289168546.33081</v>
       </c>
       <c r="D173" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E173" s="2" t="n">
+        <v>1.260163731644075</v>
       </c>
     </row>
     <row r="174">
@@ -2869,7 +3393,10 @@
         <v>3235851930.539863</v>
       </c>
       <c r="D174" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E174" s="2" t="n">
+        <v>1.936615806031017</v>
       </c>
     </row>
     <row r="175">
@@ -2883,7 +3410,10 @@
         <v>3906264047.239286</v>
       </c>
       <c r="D175" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E175" s="2" t="n">
+        <v>1.956985001390927</v>
       </c>
     </row>
     <row r="176">
@@ -2897,7 +3427,10 @@
         <v>3392982241.940281</v>
       </c>
       <c r="D176" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E176" s="2" t="n">
+        <v>1.758507820731243</v>
       </c>
     </row>
     <row r="177">
@@ -2911,7 +3444,10 @@
         <v>3322393108.150819</v>
       </c>
       <c r="D177" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E177" s="2" t="n">
+        <v>1.735146324626699</v>
       </c>
     </row>
     <row r="178">
@@ -2925,7 +3461,10 @@
         <v>2934318080.714441</v>
       </c>
       <c r="D178" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E178" s="2" t="n">
+        <v>1.681804513831122</v>
       </c>
     </row>
     <row r="179">
@@ -2939,7 +3478,10 @@
         <v>3931927124.527704</v>
       </c>
       <c r="D179" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E179" s="2" t="n">
+        <v>2.236332760276435</v>
       </c>
     </row>
     <row r="180">
@@ -2953,7 +3495,10 @@
         <v>3983440776.307714</v>
       </c>
       <c r="D180" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E180" s="2" t="n">
+        <v>2.1230371575085</v>
       </c>
     </row>
     <row r="181">
@@ -2967,7 +3512,10 @@
         <v>3364699744.205702</v>
       </c>
       <c r="D181" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E181" s="2" t="n">
+        <v>1.85189403804817</v>
       </c>
     </row>
     <row r="182">
@@ -2981,7 +3529,10 @@
         <v>2327058363.834154</v>
       </c>
       <c r="D182" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E182" s="2" t="n">
+        <v>1.288467261021343</v>
       </c>
     </row>
     <row r="183">
@@ -2995,7 +3546,10 @@
         <v>3796955976.881616</v>
       </c>
       <c r="D183" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E183" s="2" t="n">
+        <v>1.929919554718896</v>
       </c>
     </row>
     <row r="184">
@@ -3009,7 +3563,10 @@
         <v>2520326076.244194</v>
       </c>
       <c r="D184" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E184" s="2" t="n">
+        <v>1.550855033491255</v>
       </c>
     </row>
     <row r="185">
@@ -3023,7 +3580,10 @@
         <v>3029884058.829219</v>
       </c>
       <c r="D185" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E185" s="2" t="n">
+        <v>1.858030301873295</v>
       </c>
     </row>
     <row r="186">
@@ -3037,7 +3597,10 @@
         <v>3729456513.528146</v>
       </c>
       <c r="D186" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E186" s="2" t="n">
+        <v>2.130310949560251</v>
       </c>
     </row>
     <row r="187">
@@ -3053,6 +3616,9 @@
       <c r="D187" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E187" s="2" t="n">
+        <v>1.844813794992312</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="n">
@@ -3065,7 +3631,10 @@
         <v>2804512319.665326</v>
       </c>
       <c r="D188" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E188" s="2" t="n">
+        <v>1.518292529878054</v>
       </c>
     </row>
     <row r="189">
@@ -3081,6 +3650,9 @@
       <c r="D189" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E189" s="2" t="n">
+        <v>1.885102995710041</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="n">
@@ -3093,7 +3665,10 @@
         <v>2032742576.865298</v>
       </c>
       <c r="D190" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E190" s="2" t="n">
+        <v>1.508630666789234</v>
       </c>
     </row>
     <row r="191">
@@ -3107,7 +3682,10 @@
         <v>3781259648.748229</v>
       </c>
       <c r="D191" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E191" s="2" t="n">
+        <v>2.090707722705679</v>
       </c>
     </row>
     <row r="192">
@@ -3121,7 +3699,10 @@
         <v>2097095914.473666</v>
       </c>
       <c r="D192" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E192" s="2" t="n">
+        <v>1.214688579361104</v>
       </c>
     </row>
     <row r="193">
@@ -3135,7 +3716,10 @@
         <v>2312657862.752766</v>
       </c>
       <c r="D193" t="n">
-        <v>0.99</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E193" s="2" t="n">
+        <v>1.595089370991925</v>
       </c>
     </row>
     <row r="194">
@@ -3151,6 +3735,9 @@
       <c r="D194" t="n">
         <v>0.9999</v>
       </c>
+      <c r="E194" s="2" t="n">
+        <v>1.846833125702071</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="n">
@@ -3163,7 +3750,10 @@
         <v>3317412781.178983</v>
       </c>
       <c r="D195" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E195" s="2" t="n">
+        <v>1.953929175703897</v>
       </c>
     </row>
     <row r="196">
@@ -3177,7 +3767,10 @@
         <v>2480803148.562046</v>
       </c>
       <c r="D196" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E196" s="2" t="n">
+        <v>1.372572331599427</v>
       </c>
     </row>
     <row r="197">
@@ -3191,7 +3784,10 @@
         <v>2249551195.255444</v>
       </c>
       <c r="D197" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E197" s="2" t="n">
+        <v>1.429094878266814</v>
       </c>
     </row>
     <row r="198">
@@ -3205,7 +3801,10 @@
         <v>2682842651.048836</v>
       </c>
       <c r="D198" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E198" s="2" t="n">
+        <v>1.724200745539024</v>
       </c>
     </row>
     <row r="199">
@@ -3219,7 +3818,10 @@
         <v>3487561591.654347</v>
       </c>
       <c r="D199" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E199" s="2" t="n">
+        <v>1.750867739103717</v>
       </c>
     </row>
     <row r="200">
@@ -3233,7 +3835,10 @@
         <v>2512096869.018666</v>
       </c>
       <c r="D200" t="n">
-        <v>0.9</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E200" s="2" t="n">
+        <v>1.43606317215953</v>
       </c>
     </row>
     <row r="201">
@@ -3247,7 +3852,10 @@
         <v>3630904106.936749</v>
       </c>
       <c r="D201" t="n">
-        <v>0.999</v>
+        <v>0.9999</v>
+      </c>
+      <c r="E201" s="2" t="n">
+        <v>2.043471428771575</v>
       </c>
     </row>
   </sheetData>

</xml_diff>